<commit_message>
22/04/25 : début matrice de corrélation
</commit_message>
<xml_diff>
--- a/Graphiques_&_ECARTYPES_Metriques_AD.xlsx
+++ b/Graphiques_&_ECARTYPES_Metriques_AD.xlsx
@@ -24,7 +24,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="42" uniqueCount="28">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="58" uniqueCount="36">
   <si>
     <t>Ecart-type</t>
   </si>
@@ -108,6 +108,30 @@
   </si>
   <si>
     <t>10.28983</t>
+  </si>
+  <si>
+    <t>0.3272069</t>
+  </si>
+  <si>
+    <t>Metriques_TauxMortalité_Placette_AD</t>
+  </si>
+  <si>
+    <t>Metriques_Encombrement_Placette_AD</t>
+  </si>
+  <si>
+    <t>6.680769</t>
+  </si>
+  <si>
+    <t>8.363297</t>
+  </si>
+  <si>
+    <t>Metriques_DiversiteBM_Placette_AD</t>
+  </si>
+  <si>
+    <t>2.876768</t>
+  </si>
+  <si>
+    <t>Metriques_ProportionG_arbresmorts_AD</t>
   </si>
 </sst>
 </file>
@@ -673,6 +697,182 @@
     </xdr:pic>
     <xdr:clientData/>
   </xdr:twoCellAnchor>
+  <xdr:twoCellAnchor editAs="oneCell">
+    <xdr:from>
+      <xdr:col>2</xdr:col>
+      <xdr:colOff>198120</xdr:colOff>
+      <xdr:row>156</xdr:row>
+      <xdr:rowOff>152400</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>4</xdr:col>
+      <xdr:colOff>114693</xdr:colOff>
+      <xdr:row>172</xdr:row>
+      <xdr:rowOff>114552</xdr:rowOff>
+    </xdr:to>
+    <xdr:pic>
+      <xdr:nvPicPr>
+        <xdr:cNvPr id="3" name="Image 2"/>
+        <xdr:cNvPicPr>
+          <a:picLocks noChangeAspect="1"/>
+        </xdr:cNvPicPr>
+      </xdr:nvPicPr>
+      <xdr:blipFill>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId10">
+          <a:extLst>
+            <a:ext uri="{28A0092B-C50C-407E-A947-70E740481C1C}">
+              <a14:useLocalDpi xmlns:a14="http://schemas.microsoft.com/office/drawing/2010/main" val="0"/>
+            </a:ext>
+          </a:extLst>
+        </a:blip>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </xdr:blipFill>
+      <xdr:spPr>
+        <a:xfrm>
+          <a:off x="4305300" y="28864560"/>
+          <a:ext cx="4534293" cy="2911092"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+      </xdr:spPr>
+    </xdr:pic>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+  <xdr:twoCellAnchor editAs="oneCell">
+    <xdr:from>
+      <xdr:col>2</xdr:col>
+      <xdr:colOff>205740</xdr:colOff>
+      <xdr:row>173</xdr:row>
+      <xdr:rowOff>22860</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>7</xdr:col>
+      <xdr:colOff>473201</xdr:colOff>
+      <xdr:row>194</xdr:row>
+      <xdr:rowOff>99401</xdr:rowOff>
+    </xdr:to>
+    <xdr:pic>
+      <xdr:nvPicPr>
+        <xdr:cNvPr id="13" name="Image 12"/>
+        <xdr:cNvPicPr>
+          <a:picLocks noChangeAspect="1"/>
+        </xdr:cNvPicPr>
+      </xdr:nvPicPr>
+      <xdr:blipFill>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId11">
+          <a:extLst>
+            <a:ext uri="{28A0092B-C50C-407E-A947-70E740481C1C}">
+              <a14:useLocalDpi xmlns:a14="http://schemas.microsoft.com/office/drawing/2010/main" val="0"/>
+            </a:ext>
+          </a:extLst>
+        </a:blip>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </xdr:blipFill>
+      <xdr:spPr>
+        <a:xfrm>
+          <a:off x="4312920" y="31866840"/>
+          <a:ext cx="8779001" cy="3939881"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+      </xdr:spPr>
+    </xdr:pic>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+  <xdr:twoCellAnchor editAs="oneCell">
+    <xdr:from>
+      <xdr:col>2</xdr:col>
+      <xdr:colOff>289560</xdr:colOff>
+      <xdr:row>195</xdr:row>
+      <xdr:rowOff>91440</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>4</xdr:col>
+      <xdr:colOff>2157022</xdr:colOff>
+      <xdr:row>214</xdr:row>
+      <xdr:rowOff>167949</xdr:rowOff>
+    </xdr:to>
+    <xdr:pic>
+      <xdr:nvPicPr>
+        <xdr:cNvPr id="14" name="Image 13"/>
+        <xdr:cNvPicPr>
+          <a:picLocks noChangeAspect="1"/>
+        </xdr:cNvPicPr>
+      </xdr:nvPicPr>
+      <xdr:blipFill>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId12">
+          <a:extLst>
+            <a:ext uri="{28A0092B-C50C-407E-A947-70E740481C1C}">
+              <a14:useLocalDpi xmlns:a14="http://schemas.microsoft.com/office/drawing/2010/main" val="0"/>
+            </a:ext>
+          </a:extLst>
+        </a:blip>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </xdr:blipFill>
+      <xdr:spPr>
+        <a:xfrm>
+          <a:off x="4396740" y="35989260"/>
+          <a:ext cx="6485182" cy="3566469"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+      </xdr:spPr>
+    </xdr:pic>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+  <xdr:twoCellAnchor editAs="oneCell">
+    <xdr:from>
+      <xdr:col>2</xdr:col>
+      <xdr:colOff>91440</xdr:colOff>
+      <xdr:row>216</xdr:row>
+      <xdr:rowOff>38100</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>9</xdr:col>
+      <xdr:colOff>53340</xdr:colOff>
+      <xdr:row>235</xdr:row>
+      <xdr:rowOff>178239</xdr:rowOff>
+    </xdr:to>
+    <xdr:pic>
+      <xdr:nvPicPr>
+        <xdr:cNvPr id="15" name="Image 14"/>
+        <xdr:cNvPicPr>
+          <a:picLocks noChangeAspect="1"/>
+        </xdr:cNvPicPr>
+      </xdr:nvPicPr>
+      <xdr:blipFill>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId13">
+          <a:extLst>
+            <a:ext uri="{28A0092B-C50C-407E-A947-70E740481C1C}">
+              <a14:useLocalDpi xmlns:a14="http://schemas.microsoft.com/office/drawing/2010/main" val="0"/>
+            </a:ext>
+          </a:extLst>
+        </a:blip>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </xdr:blipFill>
+      <xdr:spPr>
+        <a:xfrm>
+          <a:off x="4198620" y="39799260"/>
+          <a:ext cx="10058400" cy="3630099"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+      </xdr:spPr>
+    </xdr:pic>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
 </xdr:wsDr>
 </file>
 
@@ -939,7 +1139,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:E138"/>
+  <dimension ref="A1:E218"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="49.33203125" bestFit="1" customWidth="1"/>
@@ -1140,6 +1340,74 @@
         <v>27</v>
       </c>
     </row>
+    <row r="157" spans="1:2" ht="15" thickBot="1" x14ac:dyDescent="0.35"/>
+    <row r="158" spans="1:2" ht="15" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="A158" s="6" t="s">
+        <v>8</v>
+      </c>
+      <c r="B158" s="5" t="s">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="159" spans="1:2" ht="15" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="A159" s="5" t="s">
+        <v>30</v>
+      </c>
+      <c r="B159" s="5" t="s">
+        <v>28</v>
+      </c>
+    </row>
+    <row r="174" spans="1:2" ht="15" thickBot="1" x14ac:dyDescent="0.35"/>
+    <row r="175" spans="1:2" ht="15" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="A175" s="6" t="s">
+        <v>8</v>
+      </c>
+      <c r="B175" s="5" t="s">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="176" spans="1:2" ht="15" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="A176" s="5" t="s">
+        <v>29</v>
+      </c>
+      <c r="B176" s="5" t="s">
+        <v>31</v>
+      </c>
+    </row>
+    <row r="195" spans="1:2" ht="15" thickBot="1" x14ac:dyDescent="0.35"/>
+    <row r="196" spans="1:2" ht="15" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="A196" s="6" t="s">
+        <v>8</v>
+      </c>
+      <c r="B196" s="5" t="s">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="197" spans="1:2" ht="15" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="A197" s="5" t="s">
+        <v>33</v>
+      </c>
+      <c r="B197" s="5" t="s">
+        <v>32</v>
+      </c>
+    </row>
+    <row r="216" spans="1:2" ht="15" thickBot="1" x14ac:dyDescent="0.35"/>
+    <row r="217" spans="1:2" ht="15" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="A217" s="6" t="s">
+        <v>8</v>
+      </c>
+      <c r="B217" s="5" t="s">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="218" spans="1:2" ht="15" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="A218" s="5" t="s">
+        <v>35</v>
+      </c>
+      <c r="B218" s="5" t="s">
+        <v>34</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <drawing r:id="rId1"/>

</xml_diff>

<commit_message>
23-04-25 début des corrections suite réu 22-04
</commit_message>
<xml_diff>
--- a/Graphiques_&_ECARTYPES_Metriques_AD.xlsx
+++ b/Graphiques_&_ECARTYPES_Metriques_AD.xlsx
@@ -24,7 +24,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="66" uniqueCount="45">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="114" uniqueCount="75">
   <si>
     <t>Ecart-type</t>
   </si>
@@ -134,15 +134,6 @@
     <t>Metriques_ProportionG_arbresmorts_AD</t>
   </si>
   <si>
-    <t>modif légende</t>
-  </si>
-  <si>
-    <t>Metriques__Placette_AD</t>
-  </si>
-  <si>
-    <t>refaire</t>
-  </si>
-  <si>
     <t>changer a BMP + BMD au lieu de proportions</t>
   </si>
   <si>
@@ -159,6 +150,105 @@
   </si>
   <si>
     <t>!!! Peu intéressante</t>
+  </si>
+  <si>
+    <t>Min</t>
+  </si>
+  <si>
+    <t>Max</t>
+  </si>
+  <si>
+    <t>Mean</t>
+  </si>
+  <si>
+    <t>0.1138827</t>
+  </si>
+  <si>
+    <t>0.02581996</t>
+  </si>
+  <si>
+    <t>0.08335038</t>
+  </si>
+  <si>
+    <t>0.02081305</t>
+  </si>
+  <si>
+    <t>0.4614214</t>
+  </si>
+  <si>
+    <t>0.1452987</t>
+  </si>
+  <si>
+    <t>0.003926991</t>
+  </si>
+  <si>
+    <t>0.4751659</t>
+  </si>
+  <si>
+    <t>0.1299834</t>
+  </si>
+  <si>
+    <t>38.17105</t>
+  </si>
+  <si>
+    <t>9.345811</t>
+  </si>
+  <si>
+    <t>24.44439</t>
+  </si>
+  <si>
+    <t>0.05555543</t>
+  </si>
+  <si>
+    <t>0.3351569</t>
+  </si>
+  <si>
+    <t>86.43693</t>
+  </si>
+  <si>
+    <t>27.0312</t>
+  </si>
+  <si>
+    <t>134.936</t>
+  </si>
+  <si>
+    <t>2.570209</t>
+  </si>
+  <si>
+    <t>32.19232</t>
+  </si>
+  <si>
+    <t>7.981241</t>
+  </si>
+  <si>
+    <t>0.7388666</t>
+  </si>
+  <si>
+    <t>217.9143</t>
+  </si>
+  <si>
+    <t>33.24946</t>
+  </si>
+  <si>
+    <t>2.295189</t>
+  </si>
+  <si>
+    <t>223.4094</t>
+  </si>
+  <si>
+    <t>41.2307</t>
+  </si>
+  <si>
+    <t>Metriques_BMtot_Placette_AD</t>
+  </si>
+  <si>
+    <t>14.91858</t>
+  </si>
+  <si>
+    <t>305.0853</t>
+  </si>
+  <si>
+    <t>98.4517</t>
   </si>
 </sst>
 </file>
@@ -182,7 +272,7 @@
       <patternFill patternType="gray125"/>
     </fill>
   </fills>
-  <borders count="8">
+  <borders count="16">
     <border>
       <left/>
       <right/>
@@ -289,11 +379,111 @@
       </bottom>
       <diagonal/>
     </border>
+    <border>
+      <left style="medium">
+        <color indexed="64"/>
+      </left>
+      <right/>
+      <top/>
+      <bottom style="thin">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="medium">
+        <color indexed="64"/>
+      </left>
+      <right/>
+      <top style="thin">
+        <color indexed="64"/>
+      </top>
+      <bottom style="thin">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="medium">
+        <color indexed="64"/>
+      </left>
+      <right/>
+      <top style="thin">
+        <color indexed="64"/>
+      </top>
+      <bottom style="medium">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right style="medium">
+        <color indexed="64"/>
+      </right>
+      <top style="medium">
+        <color indexed="64"/>
+      </top>
+      <bottom style="thin">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right style="medium">
+        <color indexed="64"/>
+      </right>
+      <top style="thin">
+        <color indexed="64"/>
+      </top>
+      <bottom style="thin">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right style="medium">
+        <color indexed="64"/>
+      </right>
+      <top style="thin">
+        <color indexed="64"/>
+      </top>
+      <bottom style="medium">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="medium">
+        <color indexed="64"/>
+      </left>
+      <right style="medium">
+        <color indexed="64"/>
+      </right>
+      <top/>
+      <bottom style="medium">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right style="medium">
+        <color indexed="64"/>
+      </right>
+      <top/>
+      <bottom style="medium">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="11">
+  <cellXfs count="21">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyBorder="1"/>
@@ -309,6 +499,16 @@
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="6" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="7" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="8" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="9" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="10" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="6" xfId="0" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="11" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="12" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="13" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="14" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="15" xfId="0" applyBorder="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -330,14 +530,14 @@
 <xdr:wsDr xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
   <xdr:twoCellAnchor editAs="oneCell">
     <xdr:from>
-      <xdr:col>2</xdr:col>
-      <xdr:colOff>99060</xdr:colOff>
+      <xdr:col>5</xdr:col>
+      <xdr:colOff>174943</xdr:colOff>
       <xdr:row>0</xdr:row>
       <xdr:rowOff>0</xdr:rowOff>
     </xdr:from>
     <xdr:to>
-      <xdr:col>4</xdr:col>
-      <xdr:colOff>2225039</xdr:colOff>
+      <xdr:col>13</xdr:col>
+      <xdr:colOff>570547</xdr:colOff>
       <xdr:row>21</xdr:row>
       <xdr:rowOff>145127</xdr:rowOff>
     </xdr:to>
@@ -362,8 +562,8 @@
       </xdr:blipFill>
       <xdr:spPr>
         <a:xfrm>
-          <a:off x="3131820" y="0"/>
-          <a:ext cx="6743699" cy="4000847"/>
+          <a:off x="6009006" y="0"/>
+          <a:ext cx="6745604" cy="3994815"/>
         </a:xfrm>
         <a:prstGeom prst="rect">
           <a:avLst/>
@@ -374,20 +574,20 @@
   </xdr:twoCellAnchor>
   <xdr:twoCellAnchor editAs="oneCell">
     <xdr:from>
-      <xdr:col>2</xdr:col>
-      <xdr:colOff>0</xdr:colOff>
-      <xdr:row>40</xdr:row>
-      <xdr:rowOff>0</xdr:rowOff>
+      <xdr:col>5</xdr:col>
+      <xdr:colOff>140018</xdr:colOff>
+      <xdr:row>22</xdr:row>
+      <xdr:rowOff>53022</xdr:rowOff>
     </xdr:from>
     <xdr:to>
-      <xdr:col>6</xdr:col>
-      <xdr:colOff>328357</xdr:colOff>
-      <xdr:row>59</xdr:row>
-      <xdr:rowOff>145096</xdr:rowOff>
+      <xdr:col>10</xdr:col>
+      <xdr:colOff>706513</xdr:colOff>
+      <xdr:row>38</xdr:row>
+      <xdr:rowOff>22794</xdr:rowOff>
     </xdr:to>
     <xdr:pic>
       <xdr:nvPicPr>
-        <xdr:cNvPr id="4" name="Image 3"/>
+        <xdr:cNvPr id="5" name="Image 4"/>
         <xdr:cNvPicPr>
           <a:picLocks noChangeAspect="1"/>
         </xdr:cNvPicPr>
@@ -406,8 +606,8 @@
       </xdr:blipFill>
       <xdr:spPr>
         <a:xfrm>
-          <a:off x="3169920" y="7360920"/>
-          <a:ext cx="8047417" cy="3642676"/>
+          <a:off x="6505893" y="4093210"/>
+          <a:ext cx="4535245" cy="2906647"/>
         </a:xfrm>
         <a:prstGeom prst="rect">
           <a:avLst/>
@@ -418,20 +618,20 @@
   </xdr:twoCellAnchor>
   <xdr:twoCellAnchor editAs="oneCell">
     <xdr:from>
-      <xdr:col>2</xdr:col>
-      <xdr:colOff>68580</xdr:colOff>
-      <xdr:row>22</xdr:row>
-      <xdr:rowOff>60960</xdr:rowOff>
+      <xdr:col>5</xdr:col>
+      <xdr:colOff>117793</xdr:colOff>
+      <xdr:row>70</xdr:row>
+      <xdr:rowOff>14922</xdr:rowOff>
     </xdr:from>
     <xdr:to>
-      <xdr:col>3</xdr:col>
-      <xdr:colOff>2294013</xdr:colOff>
-      <xdr:row>38</xdr:row>
-      <xdr:rowOff>30732</xdr:rowOff>
+      <xdr:col>10</xdr:col>
+      <xdr:colOff>684288</xdr:colOff>
+      <xdr:row>85</xdr:row>
+      <xdr:rowOff>159954</xdr:rowOff>
     </xdr:to>
     <xdr:pic>
       <xdr:nvPicPr>
-        <xdr:cNvPr id="5" name="Image 4"/>
+        <xdr:cNvPr id="6" name="Image 5"/>
         <xdr:cNvPicPr>
           <a:picLocks noChangeAspect="1"/>
         </xdr:cNvPicPr>
@@ -450,8 +650,8 @@
       </xdr:blipFill>
       <xdr:spPr>
         <a:xfrm>
-          <a:off x="3787140" y="4107180"/>
-          <a:ext cx="4534293" cy="2911092"/>
+          <a:off x="6483668" y="12865735"/>
+          <a:ext cx="4535245" cy="2907282"/>
         </a:xfrm>
         <a:prstGeom prst="rect">
           <a:avLst/>
@@ -462,20 +662,20 @@
   </xdr:twoCellAnchor>
   <xdr:twoCellAnchor editAs="oneCell">
     <xdr:from>
-      <xdr:col>2</xdr:col>
-      <xdr:colOff>30480</xdr:colOff>
-      <xdr:row>60</xdr:row>
-      <xdr:rowOff>22860</xdr:rowOff>
+      <xdr:col>26</xdr:col>
+      <xdr:colOff>713152</xdr:colOff>
+      <xdr:row>86</xdr:row>
+      <xdr:rowOff>87527</xdr:rowOff>
     </xdr:from>
     <xdr:to>
-      <xdr:col>3</xdr:col>
-      <xdr:colOff>2255913</xdr:colOff>
-      <xdr:row>75</xdr:row>
-      <xdr:rowOff>167892</xdr:rowOff>
+      <xdr:col>39</xdr:col>
+      <xdr:colOff>469312</xdr:colOff>
+      <xdr:row>107</xdr:row>
+      <xdr:rowOff>58534</xdr:rowOff>
     </xdr:to>
     <xdr:pic>
       <xdr:nvPicPr>
-        <xdr:cNvPr id="6" name="Image 5"/>
+        <xdr:cNvPr id="7" name="Image 6"/>
         <xdr:cNvPicPr>
           <a:picLocks noChangeAspect="1"/>
         </xdr:cNvPicPr>
@@ -494,8 +694,8 @@
       </xdr:blipFill>
       <xdr:spPr>
         <a:xfrm>
-          <a:off x="3749040" y="11064240"/>
-          <a:ext cx="4534293" cy="2911092"/>
+          <a:off x="23977965" y="15883152"/>
+          <a:ext cx="10074910" cy="3828632"/>
         </a:xfrm>
         <a:prstGeom prst="rect">
           <a:avLst/>
@@ -506,20 +706,20 @@
   </xdr:twoCellAnchor>
   <xdr:twoCellAnchor editAs="oneCell">
     <xdr:from>
-      <xdr:col>8</xdr:col>
-      <xdr:colOff>467089</xdr:colOff>
-      <xdr:row>77</xdr:row>
-      <xdr:rowOff>63715</xdr:rowOff>
+      <xdr:col>15</xdr:col>
+      <xdr:colOff>394971</xdr:colOff>
+      <xdr:row>86</xdr:row>
+      <xdr:rowOff>8890</xdr:rowOff>
     </xdr:from>
     <xdr:to>
-      <xdr:col>21</xdr:col>
-      <xdr:colOff>223249</xdr:colOff>
-      <xdr:row>98</xdr:row>
-      <xdr:rowOff>42659</xdr:rowOff>
+      <xdr:col>26</xdr:col>
+      <xdr:colOff>737704</xdr:colOff>
+      <xdr:row>108</xdr:row>
+      <xdr:rowOff>39405</xdr:rowOff>
     </xdr:to>
     <xdr:pic>
       <xdr:nvPicPr>
-        <xdr:cNvPr id="7" name="Image 6"/>
+        <xdr:cNvPr id="8" name="Image 7"/>
         <xdr:cNvPicPr>
           <a:picLocks noChangeAspect="1"/>
         </xdr:cNvPicPr>
@@ -538,8 +738,8 @@
       </xdr:blipFill>
       <xdr:spPr>
         <a:xfrm>
-          <a:off x="13883153" y="14525502"/>
-          <a:ext cx="10083692" cy="3910540"/>
+          <a:off x="14928534" y="15804515"/>
+          <a:ext cx="9073983" cy="4070703"/>
         </a:xfrm>
         <a:prstGeom prst="rect">
           <a:avLst/>
@@ -550,20 +750,20 @@
   </xdr:twoCellAnchor>
   <xdr:twoCellAnchor editAs="oneCell">
     <xdr:from>
-      <xdr:col>2</xdr:col>
-      <xdr:colOff>45720</xdr:colOff>
-      <xdr:row>76</xdr:row>
-      <xdr:rowOff>167640</xdr:rowOff>
+      <xdr:col>5</xdr:col>
+      <xdr:colOff>111125</xdr:colOff>
+      <xdr:row>108</xdr:row>
+      <xdr:rowOff>119062</xdr:rowOff>
     </xdr:from>
     <xdr:to>
-      <xdr:col>7</xdr:col>
-      <xdr:colOff>602766</xdr:colOff>
-      <xdr:row>99</xdr:row>
-      <xdr:rowOff>15593</xdr:rowOff>
+      <xdr:col>10</xdr:col>
+      <xdr:colOff>677620</xdr:colOff>
+      <xdr:row>124</xdr:row>
+      <xdr:rowOff>81215</xdr:rowOff>
     </xdr:to>
     <xdr:pic>
       <xdr:nvPicPr>
-        <xdr:cNvPr id="8" name="Image 7"/>
+        <xdr:cNvPr id="10" name="Image 9"/>
         <xdr:cNvPicPr>
           <a:picLocks noChangeAspect="1"/>
         </xdr:cNvPicPr>
@@ -582,8 +782,8 @@
       </xdr:blipFill>
       <xdr:spPr>
         <a:xfrm>
-          <a:off x="3764280" y="14157960"/>
-          <a:ext cx="9068586" cy="4077053"/>
+          <a:off x="6707188" y="19954875"/>
+          <a:ext cx="4535245" cy="2906965"/>
         </a:xfrm>
         <a:prstGeom prst="rect">
           <a:avLst/>
@@ -594,20 +794,20 @@
   </xdr:twoCellAnchor>
   <xdr:twoCellAnchor editAs="oneCell">
     <xdr:from>
-      <xdr:col>2</xdr:col>
-      <xdr:colOff>0</xdr:colOff>
-      <xdr:row>100</xdr:row>
-      <xdr:rowOff>0</xdr:rowOff>
+      <xdr:col>5</xdr:col>
+      <xdr:colOff>109219</xdr:colOff>
+      <xdr:row>126</xdr:row>
+      <xdr:rowOff>111125</xdr:rowOff>
     </xdr:from>
     <xdr:to>
-      <xdr:col>3</xdr:col>
-      <xdr:colOff>2225433</xdr:colOff>
-      <xdr:row>115</xdr:row>
-      <xdr:rowOff>152652</xdr:rowOff>
+      <xdr:col>17</xdr:col>
+      <xdr:colOff>650556</xdr:colOff>
+      <xdr:row>146</xdr:row>
+      <xdr:rowOff>20509</xdr:rowOff>
     </xdr:to>
     <xdr:pic>
       <xdr:nvPicPr>
-        <xdr:cNvPr id="10" name="Image 9"/>
+        <xdr:cNvPr id="11" name="Image 10"/>
         <xdr:cNvPicPr>
           <a:picLocks noChangeAspect="1"/>
         </xdr:cNvPicPr>
@@ -626,52 +826,8 @@
       </xdr:blipFill>
       <xdr:spPr>
         <a:xfrm>
-          <a:off x="4107180" y="18409920"/>
-          <a:ext cx="4534293" cy="2911092"/>
-        </a:xfrm>
-        <a:prstGeom prst="rect">
-          <a:avLst/>
-        </a:prstGeom>
-      </xdr:spPr>
-    </xdr:pic>
-    <xdr:clientData/>
-  </xdr:twoCellAnchor>
-  <xdr:twoCellAnchor editAs="oneCell">
-    <xdr:from>
-      <xdr:col>2</xdr:col>
-      <xdr:colOff>45720</xdr:colOff>
-      <xdr:row>116</xdr:row>
-      <xdr:rowOff>0</xdr:rowOff>
-    </xdr:from>
-    <xdr:to>
-      <xdr:col>9</xdr:col>
-      <xdr:colOff>7620</xdr:colOff>
-      <xdr:row>135</xdr:row>
-      <xdr:rowOff>99884</xdr:rowOff>
-    </xdr:to>
-    <xdr:pic>
-      <xdr:nvPicPr>
-        <xdr:cNvPr id="11" name="Image 10"/>
-        <xdr:cNvPicPr>
-          <a:picLocks noChangeAspect="1"/>
-        </xdr:cNvPicPr>
-      </xdr:nvPicPr>
-      <xdr:blipFill>
-        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId8">
-          <a:extLst>
-            <a:ext uri="{28A0092B-C50C-407E-A947-70E740481C1C}">
-              <a14:useLocalDpi xmlns:a14="http://schemas.microsoft.com/office/drawing/2010/main" val="0"/>
-            </a:ext>
-          </a:extLst>
-        </a:blip>
-        <a:stretch>
-          <a:fillRect/>
-        </a:stretch>
-      </xdr:blipFill>
-      <xdr:spPr>
-        <a:xfrm>
-          <a:off x="4152900" y="21358860"/>
-          <a:ext cx="10058400" cy="3589844"/>
+          <a:off x="6705282" y="23264813"/>
+          <a:ext cx="10066337" cy="3584446"/>
         </a:xfrm>
         <a:prstGeom prst="rect">
           <a:avLst/>
@@ -684,13 +840,13 @@
     <xdr:from>
       <xdr:col>2</xdr:col>
       <xdr:colOff>0</xdr:colOff>
-      <xdr:row>137</xdr:row>
+      <xdr:row>147</xdr:row>
       <xdr:rowOff>0</xdr:rowOff>
     </xdr:from>
     <xdr:to>
-      <xdr:col>5</xdr:col>
-      <xdr:colOff>320668</xdr:colOff>
-      <xdr:row>155</xdr:row>
+      <xdr:col>11</xdr:col>
+      <xdr:colOff>225417</xdr:colOff>
+      <xdr:row>165</xdr:row>
       <xdr:rowOff>137458</xdr:rowOff>
     </xdr:to>
     <xdr:pic>
@@ -701,7 +857,7 @@
         </xdr:cNvPicPr>
       </xdr:nvPicPr>
       <xdr:blipFill>
-        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId9">
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId8">
           <a:extLst>
             <a:ext uri="{28A0092B-C50C-407E-A947-70E740481C1C}">
               <a14:useLocalDpi xmlns:a14="http://schemas.microsoft.com/office/drawing/2010/main" val="0"/>
@@ -728,13 +884,13 @@
     <xdr:from>
       <xdr:col>2</xdr:col>
       <xdr:colOff>198120</xdr:colOff>
-      <xdr:row>156</xdr:row>
+      <xdr:row>166</xdr:row>
       <xdr:rowOff>152400</xdr:rowOff>
     </xdr:from>
     <xdr:to>
-      <xdr:col>4</xdr:col>
-      <xdr:colOff>114693</xdr:colOff>
-      <xdr:row>172</xdr:row>
+      <xdr:col>8</xdr:col>
+      <xdr:colOff>90880</xdr:colOff>
+      <xdr:row>182</xdr:row>
       <xdr:rowOff>114552</xdr:rowOff>
     </xdr:to>
     <xdr:pic>
@@ -745,7 +901,7 @@
         </xdr:cNvPicPr>
       </xdr:nvPicPr>
       <xdr:blipFill>
-        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId10">
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId9">
           <a:extLst>
             <a:ext uri="{28A0092B-C50C-407E-A947-70E740481C1C}">
               <a14:useLocalDpi xmlns:a14="http://schemas.microsoft.com/office/drawing/2010/main" val="0"/>
@@ -772,13 +928,13 @@
     <xdr:from>
       <xdr:col>2</xdr:col>
       <xdr:colOff>205740</xdr:colOff>
-      <xdr:row>173</xdr:row>
+      <xdr:row>183</xdr:row>
       <xdr:rowOff>22860</xdr:rowOff>
     </xdr:from>
     <xdr:to>
-      <xdr:col>7</xdr:col>
-      <xdr:colOff>473201</xdr:colOff>
-      <xdr:row>194</xdr:row>
+      <xdr:col>13</xdr:col>
+      <xdr:colOff>377950</xdr:colOff>
+      <xdr:row>204</xdr:row>
       <xdr:rowOff>99401</xdr:rowOff>
     </xdr:to>
     <xdr:pic>
@@ -789,7 +945,7 @@
         </xdr:cNvPicPr>
       </xdr:nvPicPr>
       <xdr:blipFill>
-        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId11">
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId10">
           <a:extLst>
             <a:ext uri="{28A0092B-C50C-407E-A947-70E740481C1C}">
               <a14:useLocalDpi xmlns:a14="http://schemas.microsoft.com/office/drawing/2010/main" val="0"/>
@@ -816,13 +972,13 @@
     <xdr:from>
       <xdr:col>2</xdr:col>
       <xdr:colOff>289560</xdr:colOff>
-      <xdr:row>195</xdr:row>
+      <xdr:row>205</xdr:row>
       <xdr:rowOff>91440</xdr:rowOff>
     </xdr:from>
     <xdr:to>
-      <xdr:col>4</xdr:col>
-      <xdr:colOff>2157022</xdr:colOff>
-      <xdr:row>214</xdr:row>
+      <xdr:col>10</xdr:col>
+      <xdr:colOff>545709</xdr:colOff>
+      <xdr:row>224</xdr:row>
       <xdr:rowOff>167949</xdr:rowOff>
     </xdr:to>
     <xdr:pic>
@@ -833,7 +989,7 @@
         </xdr:cNvPicPr>
       </xdr:nvPicPr>
       <xdr:blipFill>
-        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId12">
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId11">
           <a:extLst>
             <a:ext uri="{28A0092B-C50C-407E-A947-70E740481C1C}">
               <a14:useLocalDpi xmlns:a14="http://schemas.microsoft.com/office/drawing/2010/main" val="0"/>
@@ -860,18 +1016,62 @@
     <xdr:from>
       <xdr:col>2</xdr:col>
       <xdr:colOff>91440</xdr:colOff>
-      <xdr:row>216</xdr:row>
+      <xdr:row>226</xdr:row>
       <xdr:rowOff>38100</xdr:rowOff>
     </xdr:from>
     <xdr:to>
-      <xdr:col>9</xdr:col>
-      <xdr:colOff>53340</xdr:colOff>
-      <xdr:row>235</xdr:row>
+      <xdr:col>14</xdr:col>
+      <xdr:colOff>751839</xdr:colOff>
+      <xdr:row>245</xdr:row>
       <xdr:rowOff>178239</xdr:rowOff>
     </xdr:to>
     <xdr:pic>
       <xdr:nvPicPr>
         <xdr:cNvPr id="15" name="Image 14"/>
+        <xdr:cNvPicPr>
+          <a:picLocks noChangeAspect="1"/>
+        </xdr:cNvPicPr>
+      </xdr:nvPicPr>
+      <xdr:blipFill>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId12">
+          <a:extLst>
+            <a:ext uri="{28A0092B-C50C-407E-A947-70E740481C1C}">
+              <a14:useLocalDpi xmlns:a14="http://schemas.microsoft.com/office/drawing/2010/main" val="0"/>
+            </a:ext>
+          </a:extLst>
+        </a:blip>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </xdr:blipFill>
+      <xdr:spPr>
+        <a:xfrm>
+          <a:off x="4198620" y="39799260"/>
+          <a:ext cx="10058400" cy="3630099"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+      </xdr:spPr>
+    </xdr:pic>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+  <xdr:twoCellAnchor editAs="oneCell">
+    <xdr:from>
+      <xdr:col>11</xdr:col>
+      <xdr:colOff>0</xdr:colOff>
+      <xdr:row>22</xdr:row>
+      <xdr:rowOff>7938</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>16</xdr:col>
+      <xdr:colOff>618888</xdr:colOff>
+      <xdr:row>37</xdr:row>
+      <xdr:rowOff>164718</xdr:rowOff>
+    </xdr:to>
+    <xdr:pic>
+      <xdr:nvPicPr>
+        <xdr:cNvPr id="9" name="Image 8"/>
         <xdr:cNvPicPr>
           <a:picLocks noChangeAspect="1"/>
         </xdr:cNvPicPr>
@@ -890,8 +1090,184 @@
       </xdr:blipFill>
       <xdr:spPr>
         <a:xfrm>
-          <a:off x="4198620" y="39799260"/>
-          <a:ext cx="10058400" cy="3630099"/>
+          <a:off x="11128375" y="4048126"/>
+          <a:ext cx="4587638" cy="2911092"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+      </xdr:spPr>
+    </xdr:pic>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+  <xdr:twoCellAnchor editAs="oneCell">
+    <xdr:from>
+      <xdr:col>5</xdr:col>
+      <xdr:colOff>111125</xdr:colOff>
+      <xdr:row>39</xdr:row>
+      <xdr:rowOff>79375</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>17</xdr:col>
+      <xdr:colOff>644525</xdr:colOff>
+      <xdr:row>66</xdr:row>
+      <xdr:rowOff>147637</xdr:rowOff>
+    </xdr:to>
+    <xdr:pic>
+      <xdr:nvPicPr>
+        <xdr:cNvPr id="17" name="Image 16"/>
+        <xdr:cNvPicPr>
+          <a:picLocks noChangeAspect="1"/>
+        </xdr:cNvPicPr>
+      </xdr:nvPicPr>
+      <xdr:blipFill>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId14">
+          <a:extLst>
+            <a:ext uri="{28A0092B-C50C-407E-A947-70E740481C1C}">
+              <a14:useLocalDpi xmlns:a14="http://schemas.microsoft.com/office/drawing/2010/main" val="0"/>
+            </a:ext>
+          </a:extLst>
+        </a:blip>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </xdr:blipFill>
+      <xdr:spPr>
+        <a:xfrm>
+          <a:off x="6477000" y="7239000"/>
+          <a:ext cx="10058400" cy="5029200"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+      </xdr:spPr>
+    </xdr:pic>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+  <xdr:twoCellAnchor editAs="oneCell">
+    <xdr:from>
+      <xdr:col>11</xdr:col>
+      <xdr:colOff>7937</xdr:colOff>
+      <xdr:row>70</xdr:row>
+      <xdr:rowOff>15875</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>16</xdr:col>
+      <xdr:colOff>626825</xdr:colOff>
+      <xdr:row>85</xdr:row>
+      <xdr:rowOff>164717</xdr:rowOff>
+    </xdr:to>
+    <xdr:pic>
+      <xdr:nvPicPr>
+        <xdr:cNvPr id="18" name="Image 17"/>
+        <xdr:cNvPicPr>
+          <a:picLocks noChangeAspect="1"/>
+        </xdr:cNvPicPr>
+      </xdr:nvPicPr>
+      <xdr:blipFill>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId15">
+          <a:extLst>
+            <a:ext uri="{28A0092B-C50C-407E-A947-70E740481C1C}">
+              <a14:useLocalDpi xmlns:a14="http://schemas.microsoft.com/office/drawing/2010/main" val="0"/>
+            </a:ext>
+          </a:extLst>
+        </a:blip>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </xdr:blipFill>
+      <xdr:spPr>
+        <a:xfrm>
+          <a:off x="11136312" y="12866688"/>
+          <a:ext cx="4587638" cy="2911092"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+      </xdr:spPr>
+    </xdr:pic>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+  <xdr:twoCellAnchor editAs="oneCell">
+    <xdr:from>
+      <xdr:col>5</xdr:col>
+      <xdr:colOff>0</xdr:colOff>
+      <xdr:row>87</xdr:row>
+      <xdr:rowOff>0</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>15</xdr:col>
+      <xdr:colOff>308055</xdr:colOff>
+      <xdr:row>107</xdr:row>
+      <xdr:rowOff>74619</xdr:rowOff>
+    </xdr:to>
+    <xdr:pic>
+      <xdr:nvPicPr>
+        <xdr:cNvPr id="19" name="Image 18"/>
+        <xdr:cNvPicPr>
+          <a:picLocks noChangeAspect="1"/>
+        </xdr:cNvPicPr>
+      </xdr:nvPicPr>
+      <xdr:blipFill>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId16">
+          <a:extLst>
+            <a:ext uri="{28A0092B-C50C-407E-A947-70E740481C1C}">
+              <a14:useLocalDpi xmlns:a14="http://schemas.microsoft.com/office/drawing/2010/main" val="0"/>
+            </a:ext>
+          </a:extLst>
+        </a:blip>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </xdr:blipFill>
+      <xdr:spPr>
+        <a:xfrm>
+          <a:off x="6596063" y="15986125"/>
+          <a:ext cx="8245555" cy="3741744"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+      </xdr:spPr>
+    </xdr:pic>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+  <xdr:twoCellAnchor editAs="oneCell">
+    <xdr:from>
+      <xdr:col>10</xdr:col>
+      <xdr:colOff>722312</xdr:colOff>
+      <xdr:row>109</xdr:row>
+      <xdr:rowOff>1</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>18</xdr:col>
+      <xdr:colOff>285944</xdr:colOff>
+      <xdr:row>125</xdr:row>
+      <xdr:rowOff>141555</xdr:rowOff>
+    </xdr:to>
+    <xdr:pic>
+      <xdr:nvPicPr>
+        <xdr:cNvPr id="20" name="Image 19"/>
+        <xdr:cNvPicPr>
+          <a:picLocks noChangeAspect="1"/>
+        </xdr:cNvPicPr>
+      </xdr:nvPicPr>
+      <xdr:blipFill>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId17">
+          <a:extLst>
+            <a:ext uri="{28A0092B-C50C-407E-A947-70E740481C1C}">
+              <a14:useLocalDpi xmlns:a14="http://schemas.microsoft.com/office/drawing/2010/main" val="0"/>
+            </a:ext>
+          </a:extLst>
+        </a:blip>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </xdr:blipFill>
+      <xdr:spPr>
+        <a:xfrm>
+          <a:off x="11287125" y="20018376"/>
+          <a:ext cx="5913632" cy="3086367"/>
         </a:xfrm>
         <a:prstGeom prst="rect">
           <a:avLst/>
@@ -1166,12 +1542,14 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:E222"/>
+  <dimension ref="A1:E232"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="1" max="1" width="49.33203125" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="52.6640625" bestFit="1" customWidth="1"/>
     <col min="2" max="2" width="10.5546875" bestFit="1" customWidth="1"/>
-    <col min="3" max="5" width="33.6640625" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="12" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="10" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="11" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:5" ht="15" thickBot="1" x14ac:dyDescent="0.35">
@@ -1181,19 +1559,32 @@
       <c r="B1" s="5" t="s">
         <v>0</v>
       </c>
-      <c r="C1" s="1"/>
-      <c r="D1" s="1"/>
+      <c r="C1" s="5" t="s">
+        <v>42</v>
+      </c>
+      <c r="D1" s="5" t="s">
+        <v>43</v>
+      </c>
+      <c r="E1" s="14" t="s">
+        <v>44</v>
+      </c>
     </row>
     <row r="2" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A2" s="4" t="s">
         <v>1</v>
       </c>
-      <c r="B2" s="4" t="s">
+      <c r="B2" s="7" t="s">
         <v>4</v>
       </c>
-      <c r="C2" s="1"/>
-      <c r="D2" s="1"/>
-      <c r="E2" s="1"/>
+      <c r="C2" s="7">
+        <v>0</v>
+      </c>
+      <c r="D2" s="7" t="s">
+        <v>45</v>
+      </c>
+      <c r="E2" s="7" t="s">
+        <v>48</v>
+      </c>
     </row>
     <row r="3" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A3" s="2" t="s">
@@ -1202,9 +1593,15 @@
       <c r="B3" s="2" t="s">
         <v>5</v>
       </c>
-      <c r="C3" s="1"/>
-      <c r="D3" s="1"/>
-      <c r="E3" s="1"/>
+      <c r="C3" s="2">
+        <v>0</v>
+      </c>
+      <c r="D3" s="2" t="s">
+        <v>49</v>
+      </c>
+      <c r="E3" s="2" t="s">
+        <v>47</v>
+      </c>
     </row>
     <row r="4" spans="1:5" ht="15" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A4" s="3" t="s">
@@ -1213,270 +1610,393 @@
       <c r="B4" s="3" t="s">
         <v>6</v>
       </c>
-      <c r="C4" s="1"/>
-      <c r="D4" s="1"/>
-      <c r="E4" s="1"/>
+      <c r="C4" s="3">
+        <v>0</v>
+      </c>
+      <c r="D4" s="3" t="s">
+        <v>50</v>
+      </c>
+      <c r="E4" s="3" t="s">
+        <v>46</v>
+      </c>
     </row>
     <row r="5" spans="1:5" x14ac:dyDescent="0.3">
       <c r="C5" s="1"/>
     </row>
-    <row r="7" spans="1:5" x14ac:dyDescent="0.3">
-      <c r="A7" t="s">
-        <v>36</v>
-      </c>
-    </row>
-    <row r="22" spans="1:2" ht="15" thickBot="1" x14ac:dyDescent="0.35"/>
-    <row r="23" spans="1:2" ht="15" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="22" spans="1:5" ht="15" thickBot="1" x14ac:dyDescent="0.35"/>
+    <row r="23" spans="1:5" ht="15" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A23" s="8" t="s">
         <v>8</v>
       </c>
       <c r="B23" s="9" t="s">
         <v>0</v>
       </c>
-    </row>
-    <row r="24" spans="1:2" ht="15" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="C23" s="5" t="s">
+        <v>42</v>
+      </c>
+      <c r="D23" s="5" t="s">
+        <v>43</v>
+      </c>
+      <c r="E23" s="14" t="s">
+        <v>44</v>
+      </c>
+    </row>
+    <row r="24" spans="1:5" ht="15" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A24" s="10" t="s">
         <v>9</v>
       </c>
       <c r="B24" s="5" t="s">
         <v>10</v>
       </c>
-    </row>
-    <row r="40" spans="1:2" ht="15" thickBot="1" x14ac:dyDescent="0.35"/>
-    <row r="41" spans="1:2" ht="15" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="C24" s="5" t="s">
+        <v>51</v>
+      </c>
+      <c r="D24" s="5" t="s">
+        <v>52</v>
+      </c>
+      <c r="E24" s="5" t="s">
+        <v>53</v>
+      </c>
+    </row>
+    <row r="40" spans="1:5" ht="15" thickBot="1" x14ac:dyDescent="0.35"/>
+    <row r="41" spans="1:5" ht="15" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A41" s="8" t="s">
         <v>7</v>
       </c>
       <c r="B41" s="9" t="s">
         <v>0</v>
       </c>
-    </row>
-    <row r="42" spans="1:2" ht="15" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="C41" s="5" t="s">
+        <v>42</v>
+      </c>
+      <c r="D41" s="5" t="s">
+        <v>43</v>
+      </c>
+      <c r="E41" s="14" t="s">
+        <v>44</v>
+      </c>
+    </row>
+    <row r="42" spans="1:5" ht="15" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A42" s="10" t="s">
         <v>13</v>
       </c>
       <c r="B42" s="5" t="s">
         <v>11</v>
       </c>
-    </row>
-    <row r="43" spans="1:2" ht="15" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="C42" s="2" t="s">
+        <v>57</v>
+      </c>
+      <c r="D42" s="2" t="s">
+        <v>56</v>
+      </c>
+      <c r="E42" s="2" t="s">
+        <v>55</v>
+      </c>
+    </row>
+    <row r="43" spans="1:5" ht="15" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A43" s="10" t="s">
         <v>14</v>
       </c>
       <c r="B43" s="5" t="s">
         <v>12</v>
       </c>
-    </row>
-    <row r="61" spans="1:2" ht="15" thickBot="1" x14ac:dyDescent="0.35"/>
-    <row r="62" spans="1:2" ht="15" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="A62" s="8" t="s">
+      <c r="C43" s="3" t="s">
+        <v>58</v>
+      </c>
+      <c r="D43" s="3" t="s">
+        <v>59</v>
+      </c>
+      <c r="E43" s="3" t="s">
+        <v>54</v>
+      </c>
+    </row>
+    <row r="71" spans="1:5" ht="15" thickBot="1" x14ac:dyDescent="0.35"/>
+    <row r="72" spans="1:5" ht="15" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="A72" s="8" t="s">
         <v>8</v>
       </c>
-      <c r="B62" s="9" t="s">
+      <c r="B72" s="9" t="s">
         <v>0</v>
       </c>
-    </row>
-    <row r="63" spans="1:2" ht="15" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="A63" s="10" t="s">
+      <c r="C72" s="5" t="s">
+        <v>42</v>
+      </c>
+      <c r="D72" s="5" t="s">
+        <v>43</v>
+      </c>
+      <c r="E72" s="14" t="s">
+        <v>44</v>
+      </c>
+    </row>
+    <row r="73" spans="1:5" ht="15" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="A73" s="10" t="s">
         <v>16</v>
       </c>
-      <c r="B63" s="5" t="s">
+      <c r="B73" s="5" t="s">
         <v>15</v>
       </c>
-    </row>
-    <row r="64" spans="1:2" x14ac:dyDescent="0.3">
-      <c r="A64" s="1"/>
-      <c r="B64" s="1"/>
-    </row>
-    <row r="77" spans="1:2" ht="15" thickBot="1" x14ac:dyDescent="0.35"/>
-    <row r="78" spans="1:2" ht="15" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="A78" s="6" t="s">
+      <c r="C73" s="3" t="s">
+        <v>62</v>
+      </c>
+      <c r="D73" s="3" t="s">
+        <v>61</v>
+      </c>
+      <c r="E73" s="3" t="s">
+        <v>60</v>
+      </c>
+    </row>
+    <row r="74" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A74" s="1"/>
+      <c r="B74" s="1"/>
+    </row>
+    <row r="87" spans="1:5" ht="15" thickBot="1" x14ac:dyDescent="0.35"/>
+    <row r="88" spans="1:5" ht="15" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="A88" s="6" t="s">
         <v>7</v>
       </c>
-      <c r="B78" s="5" t="s">
+      <c r="B88" s="5" t="s">
         <v>0</v>
       </c>
-    </row>
-    <row r="79" spans="1:2" x14ac:dyDescent="0.3">
-      <c r="A79" s="7" t="s">
+      <c r="C88" s="9" t="s">
+        <v>42</v>
+      </c>
+      <c r="D88" s="9" t="s">
+        <v>43</v>
+      </c>
+      <c r="E88" s="15" t="s">
+        <v>44</v>
+      </c>
+    </row>
+    <row r="89" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A89" s="7" t="s">
         <v>22</v>
       </c>
-      <c r="B79" s="4" t="s">
+      <c r="B89" s="11" t="s">
         <v>17</v>
       </c>
-    </row>
-    <row r="80" spans="1:2" x14ac:dyDescent="0.3">
-      <c r="A80" s="2" t="s">
+      <c r="C89" s="7">
+        <v>0</v>
+      </c>
+      <c r="D89" s="7" t="s">
+        <v>63</v>
+      </c>
+      <c r="E89" s="16" t="s">
+        <v>64</v>
+      </c>
+    </row>
+    <row r="90" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A90" s="2" t="s">
         <v>23</v>
       </c>
-      <c r="B80" s="2" t="s">
+      <c r="B90" s="12" t="s">
         <v>18</v>
       </c>
-    </row>
-    <row r="81" spans="1:2" ht="15" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="A81" s="3" t="s">
+      <c r="C90" s="2" t="s">
+        <v>65</v>
+      </c>
+      <c r="D90" s="2" t="s">
+        <v>66</v>
+      </c>
+      <c r="E90" s="17" t="s">
+        <v>67</v>
+      </c>
+    </row>
+    <row r="91" spans="1:5" ht="15" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="A91" s="3" t="s">
         <v>24</v>
       </c>
-      <c r="B81" s="3" t="s">
+      <c r="B91" s="13" t="s">
         <v>19</v>
       </c>
-    </row>
-    <row r="100" spans="1:2" ht="15" thickBot="1" x14ac:dyDescent="0.35"/>
-    <row r="101" spans="1:2" ht="15" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="A101" s="6" t="s">
+      <c r="C91" s="3" t="s">
+        <v>68</v>
+      </c>
+      <c r="D91" s="3" t="s">
+        <v>69</v>
+      </c>
+      <c r="E91" s="18" t="s">
+        <v>70</v>
+      </c>
+    </row>
+    <row r="110" spans="1:5" ht="15" thickBot="1" x14ac:dyDescent="0.35"/>
+    <row r="111" spans="1:5" ht="15" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="A111" s="6" t="s">
         <v>8</v>
       </c>
-      <c r="B101" s="5" t="s">
+      <c r="B111" s="5" t="s">
         <v>0</v>
       </c>
-    </row>
-    <row r="102" spans="1:2" ht="15" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="A102" s="5" t="s">
+      <c r="C111" s="5" t="s">
+        <v>42</v>
+      </c>
+      <c r="D111" s="5" t="s">
+        <v>43</v>
+      </c>
+      <c r="E111" s="14" t="s">
+        <v>44</v>
+      </c>
+    </row>
+    <row r="112" spans="1:5" ht="15" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="A112" s="5" t="s">
+        <v>71</v>
+      </c>
+      <c r="B112" s="5" t="s">
+        <v>25</v>
+      </c>
+      <c r="C112" s="19" t="s">
+        <v>72</v>
+      </c>
+      <c r="D112" s="19" t="s">
+        <v>73</v>
+      </c>
+      <c r="E112" s="20" t="s">
+        <v>74</v>
+      </c>
+    </row>
+    <row r="126" spans="1:5" ht="15" thickBot="1" x14ac:dyDescent="0.35"/>
+    <row r="127" spans="1:5" ht="15" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="A127" s="6" t="s">
+        <v>8</v>
+      </c>
+      <c r="B127" s="5" t="s">
+        <v>0</v>
+      </c>
+      <c r="C127" s="5" t="s">
+        <v>42</v>
+      </c>
+      <c r="D127" s="5" t="s">
+        <v>43</v>
+      </c>
+      <c r="E127" s="14" t="s">
+        <v>44</v>
+      </c>
+    </row>
+    <row r="128" spans="1:5" ht="15" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="A128" s="5" t="s">
+        <v>21</v>
+      </c>
+      <c r="B128" s="5" t="s">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="133" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="A133" t="s">
+        <v>36</v>
+      </c>
+    </row>
+    <row r="146" spans="1:2" ht="15" thickBot="1" x14ac:dyDescent="0.35"/>
+    <row r="147" spans="1:2" ht="15" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="A147" s="6" t="s">
+        <v>8</v>
+      </c>
+      <c r="B147" s="5" t="s">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="148" spans="1:2" ht="15" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="A148" s="5" t="s">
+        <v>26</v>
+      </c>
+      <c r="B148" s="5" t="s">
+        <v>27</v>
+      </c>
+    </row>
+    <row r="167" spans="1:2" ht="15" thickBot="1" x14ac:dyDescent="0.35"/>
+    <row r="168" spans="1:2" ht="15" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="A168" s="6" t="s">
+        <v>8</v>
+      </c>
+      <c r="B168" s="5" t="s">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="169" spans="1:2" ht="15" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="A169" s="5" t="s">
+        <v>30</v>
+      </c>
+      <c r="B169" s="5" t="s">
+        <v>28</v>
+      </c>
+    </row>
+    <row r="174" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A174" t="s">
         <v>37</v>
       </c>
-      <c r="B102" s="5" t="s">
-        <v>25</v>
-      </c>
-    </row>
-    <row r="104" spans="1:2" x14ac:dyDescent="0.3">
-      <c r="A104" t="s">
+    </row>
+    <row r="184" spans="1:2" ht="15" thickBot="1" x14ac:dyDescent="0.35"/>
+    <row r="185" spans="1:2" ht="15" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="A185" s="6" t="s">
+        <v>8</v>
+      </c>
+      <c r="B185" s="5" t="s">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="186" spans="1:2" ht="15" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="A186" s="5" t="s">
+        <v>29</v>
+      </c>
+      <c r="B186" s="5" t="s">
+        <v>31</v>
+      </c>
+    </row>
+    <row r="205" spans="1:2" ht="15" thickBot="1" x14ac:dyDescent="0.35"/>
+    <row r="206" spans="1:2" ht="15" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="A206" s="6" t="s">
+        <v>8</v>
+      </c>
+      <c r="B206" s="5" t="s">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="207" spans="1:2" ht="15" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="A207" s="5" t="s">
+        <v>33</v>
+      </c>
+      <c r="B207" s="5" t="s">
+        <v>32</v>
+      </c>
+    </row>
+    <row r="212" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="A212" t="s">
         <v>38</v>
       </c>
     </row>
-    <row r="116" spans="1:2" ht="15" thickBot="1" x14ac:dyDescent="0.35"/>
-    <row r="117" spans="1:2" ht="15" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="A117" s="6" t="s">
+    <row r="213" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="A213" t="s">
+        <v>39</v>
+      </c>
+    </row>
+    <row r="214" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="A214" t="s">
+        <v>40</v>
+      </c>
+    </row>
+    <row r="226" spans="1:2" ht="15" thickBot="1" x14ac:dyDescent="0.35"/>
+    <row r="227" spans="1:2" ht="15" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="A227" s="6" t="s">
         <v>8</v>
       </c>
-      <c r="B117" s="5" t="s">
+      <c r="B227" s="5" t="s">
         <v>0</v>
       </c>
     </row>
-    <row r="118" spans="1:2" ht="15" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="A118" s="5" t="s">
-        <v>21</v>
-      </c>
-      <c r="B118" s="5" t="s">
-        <v>20</v>
-      </c>
-    </row>
-    <row r="123" spans="1:2" x14ac:dyDescent="0.3">
-      <c r="A123" t="s">
-        <v>39</v>
-      </c>
-    </row>
-    <row r="136" spans="1:2" ht="15" thickBot="1" x14ac:dyDescent="0.35"/>
-    <row r="137" spans="1:2" ht="15" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="A137" s="6" t="s">
-        <v>8</v>
-      </c>
-      <c r="B137" s="5" t="s">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="138" spans="1:2" ht="15" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="A138" s="5" t="s">
-        <v>26</v>
-      </c>
-      <c r="B138" s="5" t="s">
-        <v>27</v>
-      </c>
-    </row>
-    <row r="157" spans="1:2" ht="15" thickBot="1" x14ac:dyDescent="0.35"/>
-    <row r="158" spans="1:2" ht="15" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="A158" s="6" t="s">
-        <v>8</v>
-      </c>
-      <c r="B158" s="5" t="s">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="159" spans="1:2" ht="15" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="A159" s="5" t="s">
-        <v>30</v>
-      </c>
-      <c r="B159" s="5" t="s">
-        <v>28</v>
-      </c>
-    </row>
-    <row r="164" spans="1:2" x14ac:dyDescent="0.3">
-      <c r="A164" t="s">
-        <v>40</v>
-      </c>
-    </row>
-    <row r="174" spans="1:2" ht="15" thickBot="1" x14ac:dyDescent="0.35"/>
-    <row r="175" spans="1:2" ht="15" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="A175" s="6" t="s">
-        <v>8</v>
-      </c>
-      <c r="B175" s="5" t="s">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="176" spans="1:2" ht="15" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="A176" s="5" t="s">
-        <v>29</v>
-      </c>
-      <c r="B176" s="5" t="s">
-        <v>31</v>
-      </c>
-    </row>
-    <row r="195" spans="1:2" ht="15" thickBot="1" x14ac:dyDescent="0.35"/>
-    <row r="196" spans="1:2" ht="15" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="A196" s="6" t="s">
-        <v>8</v>
-      </c>
-      <c r="B196" s="5" t="s">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="197" spans="1:2" ht="15" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="A197" s="5" t="s">
-        <v>33</v>
-      </c>
-      <c r="B197" s="5" t="s">
-        <v>32</v>
-      </c>
-    </row>
-    <row r="202" spans="1:2" x14ac:dyDescent="0.3">
-      <c r="A202" t="s">
+    <row r="228" spans="1:2" ht="15" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="A228" s="5" t="s">
+        <v>35</v>
+      </c>
+      <c r="B228" s="5" t="s">
+        <v>34</v>
+      </c>
+    </row>
+    <row r="232" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A232" t="s">
         <v>41</v>
-      </c>
-    </row>
-    <row r="203" spans="1:2" x14ac:dyDescent="0.3">
-      <c r="A203" t="s">
-        <v>42</v>
-      </c>
-    </row>
-    <row r="204" spans="1:2" x14ac:dyDescent="0.3">
-      <c r="A204" t="s">
-        <v>43</v>
-      </c>
-    </row>
-    <row r="216" spans="1:2" ht="15" thickBot="1" x14ac:dyDescent="0.35"/>
-    <row r="217" spans="1:2" ht="15" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="A217" s="6" t="s">
-        <v>8</v>
-      </c>
-      <c r="B217" s="5" t="s">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="218" spans="1:2" ht="15" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="A218" s="5" t="s">
-        <v>35</v>
-      </c>
-      <c r="B218" s="5" t="s">
-        <v>34</v>
-      </c>
-    </row>
-    <row r="222" spans="1:2" x14ac:dyDescent="0.3">
-      <c r="A222" t="s">
-        <v>44</v>
       </c>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <drawing r:id="rId1"/>
+  <pageSetup paperSize="9" orientation="portrait" r:id="rId1"/>
+  <drawing r:id="rId2"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
25-04-25 : fin métriques div bm et début filtrage de la matrice de corrélation
</commit_message>
<xml_diff>
--- a/Graphiques_&_ECARTYPES_Metriques_AD.xlsx
+++ b/Graphiques_&_ECARTYPES_Metriques_AD.xlsx
@@ -24,7 +24,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="114" uniqueCount="75">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="145" uniqueCount="94">
   <si>
     <t>Ecart-type</t>
   </si>
@@ -86,12 +86,6 @@
     <t>50.10593</t>
   </si>
   <si>
-    <t>15.4584</t>
-  </si>
-  <si>
-    <t>Metriques_ProportionBM_Placette_AD</t>
-  </si>
-  <si>
     <t>Metriques_BMDtot_Placette_AD : Chandelles</t>
   </si>
   <si>
@@ -110,36 +104,18 @@
     <t>10.28983</t>
   </si>
   <si>
-    <t>0.3272069</t>
-  </si>
-  <si>
     <t>Metriques_TauxMortalité_Placette_AD</t>
   </si>
   <si>
-    <t>Metriques_Encombrement_Placette_AD</t>
-  </si>
-  <si>
     <t>6.680769</t>
   </si>
   <si>
-    <t>8.363297</t>
-  </si>
-  <si>
-    <t>Metriques_DiversiteBM_Placette_AD</t>
-  </si>
-  <si>
     <t>2.876768</t>
   </si>
   <si>
     <t>Metriques_ProportionG_arbresmorts_AD</t>
   </si>
   <si>
-    <t>changer a BMP + BMD au lieu de proportions</t>
-  </si>
-  <si>
-    <t>faire métrique encombrement totale (additif)</t>
-  </si>
-  <si>
     <t>classe de diamètre a redéfinir : ex : petit (5-15cm)</t>
   </si>
   <si>
@@ -249,6 +225,87 @@
   </si>
   <si>
     <t>98.4517</t>
+  </si>
+  <si>
+    <t>55.70878</t>
+  </si>
+  <si>
+    <t>6.950929</t>
+  </si>
+  <si>
+    <t>259.8496</t>
+  </si>
+  <si>
+    <t>71.42051</t>
+  </si>
+  <si>
+    <t>Metriques_Vol_BMP&amp;BMD_Placette_AD</t>
+  </si>
+  <si>
+    <t>Anciennement</t>
+  </si>
+  <si>
+    <t>0.65</t>
+  </si>
+  <si>
+    <t>45.11</t>
+  </si>
+  <si>
+    <t>14.144</t>
+  </si>
+  <si>
+    <t>Metriques_Encombrement_Placette_AD : understory</t>
+  </si>
+  <si>
+    <t>Metriques_Encombrement_Placette_AD : canopy</t>
+  </si>
+  <si>
+    <t>3.2</t>
+  </si>
+  <si>
+    <t>6.1</t>
+  </si>
+  <si>
+    <t>2.504732</t>
+  </si>
+  <si>
+    <t>1.860956</t>
+  </si>
+  <si>
+    <t>7.411021</t>
+  </si>
+  <si>
+    <t>21.73913</t>
+  </si>
+  <si>
+    <t>1.25</t>
+  </si>
+  <si>
+    <t>21.15</t>
+  </si>
+  <si>
+    <t>5.412218</t>
+  </si>
+  <si>
+    <t>2.459191</t>
+  </si>
+  <si>
+    <t>4.380952</t>
+  </si>
+  <si>
+    <t>6.982632</t>
+  </si>
+  <si>
+    <t>19.57143</t>
+  </si>
+  <si>
+    <t>Metriques_DiversiteBM_Placette_AD : canopée</t>
+  </si>
+  <si>
+    <t>Metriques_DiversiteBM_Placette_AD : sous-étage</t>
+  </si>
+  <si>
+    <t>Metriques_DiversiteBM_Placette_AD : échelle placette</t>
   </si>
 </sst>
 </file>
@@ -264,15 +321,21 @@
       <scheme val="minor"/>
     </font>
   </fonts>
-  <fills count="2">
+  <fills count="3">
     <fill>
       <patternFill patternType="none"/>
     </fill>
     <fill>
       <patternFill patternType="gray125"/>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FF92D050"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
   </fills>
-  <borders count="16">
+  <borders count="17">
     <border>
       <left/>
       <right/>
@@ -479,11 +542,22 @@
       </bottom>
       <diagonal/>
     </border>
+    <border>
+      <left/>
+      <right style="medium">
+        <color indexed="64"/>
+      </right>
+      <top/>
+      <bottom style="thin">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="21">
+  <cellXfs count="23">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyBorder="1"/>
@@ -509,6 +583,8 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="13" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="14" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="15" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="16" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -713,7 +789,7 @@
     </xdr:from>
     <xdr:to>
       <xdr:col>26</xdr:col>
-      <xdr:colOff>737704</xdr:colOff>
+      <xdr:colOff>626579</xdr:colOff>
       <xdr:row>108</xdr:row>
       <xdr:rowOff>39405</xdr:rowOff>
     </xdr:to>
@@ -794,16 +870,16 @@
   </xdr:twoCellAnchor>
   <xdr:twoCellAnchor editAs="oneCell">
     <xdr:from>
-      <xdr:col>5</xdr:col>
-      <xdr:colOff>109219</xdr:colOff>
+      <xdr:col>18</xdr:col>
+      <xdr:colOff>514032</xdr:colOff>
       <xdr:row>126</xdr:row>
-      <xdr:rowOff>111125</xdr:rowOff>
+      <xdr:rowOff>23813</xdr:rowOff>
     </xdr:from>
     <xdr:to>
-      <xdr:col>17</xdr:col>
-      <xdr:colOff>650556</xdr:colOff>
-      <xdr:row>146</xdr:row>
-      <xdr:rowOff>20509</xdr:rowOff>
+      <xdr:col>31</xdr:col>
+      <xdr:colOff>261619</xdr:colOff>
+      <xdr:row>145</xdr:row>
+      <xdr:rowOff>123697</xdr:rowOff>
     </xdr:to>
     <xdr:pic>
       <xdr:nvPicPr>
@@ -826,7 +902,7 @@
       </xdr:blipFill>
       <xdr:spPr>
         <a:xfrm>
-          <a:off x="6705282" y="23264813"/>
+          <a:off x="17428845" y="23177501"/>
           <a:ext cx="10066337" cy="3584446"/>
         </a:xfrm>
         <a:prstGeom prst="rect">
@@ -838,16 +914,16 @@
   </xdr:twoCellAnchor>
   <xdr:twoCellAnchor editAs="oneCell">
     <xdr:from>
-      <xdr:col>2</xdr:col>
-      <xdr:colOff>0</xdr:colOff>
-      <xdr:row>147</xdr:row>
-      <xdr:rowOff>0</xdr:rowOff>
+      <xdr:col>14</xdr:col>
+      <xdr:colOff>460375</xdr:colOff>
+      <xdr:row>146</xdr:row>
+      <xdr:rowOff>39687</xdr:rowOff>
     </xdr:from>
     <xdr:to>
-      <xdr:col>11</xdr:col>
-      <xdr:colOff>225417</xdr:colOff>
-      <xdr:row>165</xdr:row>
-      <xdr:rowOff>137458</xdr:rowOff>
+      <xdr:col>23</xdr:col>
+      <xdr:colOff>455605</xdr:colOff>
+      <xdr:row>164</xdr:row>
+      <xdr:rowOff>169208</xdr:rowOff>
     </xdr:to>
     <xdr:pic>
       <xdr:nvPicPr>
@@ -870,140 +946,8 @@
       </xdr:blipFill>
       <xdr:spPr>
         <a:xfrm>
-          <a:off x="4107180" y="25214580"/>
-          <a:ext cx="7247248" cy="3436918"/>
-        </a:xfrm>
-        <a:prstGeom prst="rect">
-          <a:avLst/>
-        </a:prstGeom>
-      </xdr:spPr>
-    </xdr:pic>
-    <xdr:clientData/>
-  </xdr:twoCellAnchor>
-  <xdr:twoCellAnchor editAs="oneCell">
-    <xdr:from>
-      <xdr:col>2</xdr:col>
-      <xdr:colOff>198120</xdr:colOff>
-      <xdr:row>166</xdr:row>
-      <xdr:rowOff>152400</xdr:rowOff>
-    </xdr:from>
-    <xdr:to>
-      <xdr:col>8</xdr:col>
-      <xdr:colOff>90880</xdr:colOff>
-      <xdr:row>182</xdr:row>
-      <xdr:rowOff>114552</xdr:rowOff>
-    </xdr:to>
-    <xdr:pic>
-      <xdr:nvPicPr>
-        <xdr:cNvPr id="3" name="Image 2"/>
-        <xdr:cNvPicPr>
-          <a:picLocks noChangeAspect="1"/>
-        </xdr:cNvPicPr>
-      </xdr:nvPicPr>
-      <xdr:blipFill>
-        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId9">
-          <a:extLst>
-            <a:ext uri="{28A0092B-C50C-407E-A947-70E740481C1C}">
-              <a14:useLocalDpi xmlns:a14="http://schemas.microsoft.com/office/drawing/2010/main" val="0"/>
-            </a:ext>
-          </a:extLst>
-        </a:blip>
-        <a:stretch>
-          <a:fillRect/>
-        </a:stretch>
-      </xdr:blipFill>
-      <xdr:spPr>
-        <a:xfrm>
-          <a:off x="4305300" y="28864560"/>
-          <a:ext cx="4534293" cy="2911092"/>
-        </a:xfrm>
-        <a:prstGeom prst="rect">
-          <a:avLst/>
-        </a:prstGeom>
-      </xdr:spPr>
-    </xdr:pic>
-    <xdr:clientData/>
-  </xdr:twoCellAnchor>
-  <xdr:twoCellAnchor editAs="oneCell">
-    <xdr:from>
-      <xdr:col>2</xdr:col>
-      <xdr:colOff>205740</xdr:colOff>
-      <xdr:row>183</xdr:row>
-      <xdr:rowOff>22860</xdr:rowOff>
-    </xdr:from>
-    <xdr:to>
-      <xdr:col>13</xdr:col>
-      <xdr:colOff>377950</xdr:colOff>
-      <xdr:row>204</xdr:row>
-      <xdr:rowOff>99401</xdr:rowOff>
-    </xdr:to>
-    <xdr:pic>
-      <xdr:nvPicPr>
-        <xdr:cNvPr id="13" name="Image 12"/>
-        <xdr:cNvPicPr>
-          <a:picLocks noChangeAspect="1"/>
-        </xdr:cNvPicPr>
-      </xdr:nvPicPr>
-      <xdr:blipFill>
-        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId10">
-          <a:extLst>
-            <a:ext uri="{28A0092B-C50C-407E-A947-70E740481C1C}">
-              <a14:useLocalDpi xmlns:a14="http://schemas.microsoft.com/office/drawing/2010/main" val="0"/>
-            </a:ext>
-          </a:extLst>
-        </a:blip>
-        <a:stretch>
-          <a:fillRect/>
-        </a:stretch>
-      </xdr:blipFill>
-      <xdr:spPr>
-        <a:xfrm>
-          <a:off x="4312920" y="31866840"/>
-          <a:ext cx="8779001" cy="3939881"/>
-        </a:xfrm>
-        <a:prstGeom prst="rect">
-          <a:avLst/>
-        </a:prstGeom>
-      </xdr:spPr>
-    </xdr:pic>
-    <xdr:clientData/>
-  </xdr:twoCellAnchor>
-  <xdr:twoCellAnchor editAs="oneCell">
-    <xdr:from>
-      <xdr:col>2</xdr:col>
-      <xdr:colOff>289560</xdr:colOff>
-      <xdr:row>205</xdr:row>
-      <xdr:rowOff>91440</xdr:rowOff>
-    </xdr:from>
-    <xdr:to>
-      <xdr:col>10</xdr:col>
-      <xdr:colOff>545709</xdr:colOff>
-      <xdr:row>224</xdr:row>
-      <xdr:rowOff>167949</xdr:rowOff>
-    </xdr:to>
-    <xdr:pic>
-      <xdr:nvPicPr>
-        <xdr:cNvPr id="14" name="Image 13"/>
-        <xdr:cNvPicPr>
-          <a:picLocks noChangeAspect="1"/>
-        </xdr:cNvPicPr>
-      </xdr:nvPicPr>
-      <xdr:blipFill>
-        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId11">
-          <a:extLst>
-            <a:ext uri="{28A0092B-C50C-407E-A947-70E740481C1C}">
-              <a14:useLocalDpi xmlns:a14="http://schemas.microsoft.com/office/drawing/2010/main" val="0"/>
-            </a:ext>
-          </a:extLst>
-        </a:blip>
-        <a:stretch>
-          <a:fillRect/>
-        </a:stretch>
-      </xdr:blipFill>
-      <xdr:spPr>
-        <a:xfrm>
-          <a:off x="4396740" y="35989260"/>
-          <a:ext cx="6485182" cy="3566469"/>
+          <a:off x="14200188" y="26868437"/>
+          <a:ext cx="7250105" cy="3431521"/>
         </a:xfrm>
         <a:prstGeom prst="rect">
           <a:avLst/>
@@ -1033,7 +977,7 @@
         </xdr:cNvPicPr>
       </xdr:nvPicPr>
       <xdr:blipFill>
-        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId12">
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId9">
           <a:extLst>
             <a:ext uri="{28A0092B-C50C-407E-A947-70E740481C1C}">
               <a14:useLocalDpi xmlns:a14="http://schemas.microsoft.com/office/drawing/2010/main" val="0"/>
@@ -1077,7 +1021,7 @@
         </xdr:cNvPicPr>
       </xdr:nvPicPr>
       <xdr:blipFill>
-        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId13">
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId10">
           <a:extLst>
             <a:ext uri="{28A0092B-C50C-407E-A947-70E740481C1C}">
               <a14:useLocalDpi xmlns:a14="http://schemas.microsoft.com/office/drawing/2010/main" val="0"/>
@@ -1121,7 +1065,7 @@
         </xdr:cNvPicPr>
       </xdr:nvPicPr>
       <xdr:blipFill>
-        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId14">
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId11">
           <a:extLst>
             <a:ext uri="{28A0092B-C50C-407E-A947-70E740481C1C}">
               <a14:useLocalDpi xmlns:a14="http://schemas.microsoft.com/office/drawing/2010/main" val="0"/>
@@ -1165,7 +1109,7 @@
         </xdr:cNvPicPr>
       </xdr:nvPicPr>
       <xdr:blipFill>
-        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId15">
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId12">
           <a:extLst>
             <a:ext uri="{28A0092B-C50C-407E-A947-70E740481C1C}">
               <a14:useLocalDpi xmlns:a14="http://schemas.microsoft.com/office/drawing/2010/main" val="0"/>
@@ -1209,7 +1153,7 @@
         </xdr:cNvPicPr>
       </xdr:nvPicPr>
       <xdr:blipFill>
-        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId16">
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId13">
           <a:extLst>
             <a:ext uri="{28A0092B-C50C-407E-A947-70E740481C1C}">
               <a14:useLocalDpi xmlns:a14="http://schemas.microsoft.com/office/drawing/2010/main" val="0"/>
@@ -1235,19 +1179,151 @@
   <xdr:twoCellAnchor editAs="oneCell">
     <xdr:from>
       <xdr:col>10</xdr:col>
-      <xdr:colOff>722312</xdr:colOff>
-      <xdr:row>109</xdr:row>
-      <xdr:rowOff>1</xdr:rowOff>
+      <xdr:colOff>762000</xdr:colOff>
+      <xdr:row>108</xdr:row>
+      <xdr:rowOff>47626</xdr:rowOff>
     </xdr:from>
     <xdr:to>
       <xdr:col>18</xdr:col>
-      <xdr:colOff>285944</xdr:colOff>
+      <xdr:colOff>214507</xdr:colOff>
       <xdr:row>125</xdr:row>
-      <xdr:rowOff>141555</xdr:rowOff>
+      <xdr:rowOff>6618</xdr:rowOff>
     </xdr:to>
     <xdr:pic>
       <xdr:nvPicPr>
         <xdr:cNvPr id="20" name="Image 19"/>
+        <xdr:cNvPicPr>
+          <a:picLocks noChangeAspect="1"/>
+        </xdr:cNvPicPr>
+      </xdr:nvPicPr>
+      <xdr:blipFill>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId14">
+          <a:extLst>
+            <a:ext uri="{28A0092B-C50C-407E-A947-70E740481C1C}">
+              <a14:useLocalDpi xmlns:a14="http://schemas.microsoft.com/office/drawing/2010/main" val="0"/>
+            </a:ext>
+          </a:extLst>
+        </a:blip>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </xdr:blipFill>
+      <xdr:spPr>
+        <a:xfrm>
+          <a:off x="11326813" y="19883439"/>
+          <a:ext cx="5913632" cy="3086367"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+      </xdr:spPr>
+    </xdr:pic>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+  <xdr:twoCellAnchor editAs="oneCell">
+    <xdr:from>
+      <xdr:col>5</xdr:col>
+      <xdr:colOff>182563</xdr:colOff>
+      <xdr:row>126</xdr:row>
+      <xdr:rowOff>23812</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>13</xdr:col>
+      <xdr:colOff>211056</xdr:colOff>
+      <xdr:row>143</xdr:row>
+      <xdr:rowOff>66949</xdr:rowOff>
+    </xdr:to>
+    <xdr:pic>
+      <xdr:nvPicPr>
+        <xdr:cNvPr id="4" name="Image 3"/>
+        <xdr:cNvPicPr>
+          <a:picLocks noChangeAspect="1"/>
+        </xdr:cNvPicPr>
+      </xdr:nvPicPr>
+      <xdr:blipFill>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId15">
+          <a:extLst>
+            <a:ext uri="{28A0092B-C50C-407E-A947-70E740481C1C}">
+              <a14:useLocalDpi xmlns:a14="http://schemas.microsoft.com/office/drawing/2010/main" val="0"/>
+            </a:ext>
+          </a:extLst>
+        </a:blip>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </xdr:blipFill>
+      <xdr:spPr>
+        <a:xfrm>
+          <a:off x="6778626" y="23177500"/>
+          <a:ext cx="6378493" cy="3162574"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+      </xdr:spPr>
+    </xdr:pic>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+  <xdr:twoCellAnchor editAs="oneCell">
+    <xdr:from>
+      <xdr:col>5</xdr:col>
+      <xdr:colOff>404812</xdr:colOff>
+      <xdr:row>146</xdr:row>
+      <xdr:rowOff>55562</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>14</xdr:col>
+      <xdr:colOff>500689</xdr:colOff>
+      <xdr:row>164</xdr:row>
+      <xdr:rowOff>83791</xdr:rowOff>
+    </xdr:to>
+    <xdr:pic>
+      <xdr:nvPicPr>
+        <xdr:cNvPr id="16" name="Image 15"/>
+        <xdr:cNvPicPr>
+          <a:picLocks noChangeAspect="1"/>
+        </xdr:cNvPicPr>
+      </xdr:nvPicPr>
+      <xdr:blipFill>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId16">
+          <a:extLst>
+            <a:ext uri="{28A0092B-C50C-407E-A947-70E740481C1C}">
+              <a14:useLocalDpi xmlns:a14="http://schemas.microsoft.com/office/drawing/2010/main" val="0"/>
+            </a:ext>
+          </a:extLst>
+        </a:blip>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </xdr:blipFill>
+      <xdr:spPr>
+        <a:xfrm>
+          <a:off x="7000875" y="26884312"/>
+          <a:ext cx="7239627" cy="3330229"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+      </xdr:spPr>
+    </xdr:pic>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+  <xdr:twoCellAnchor editAs="oneCell">
+    <xdr:from>
+      <xdr:col>5</xdr:col>
+      <xdr:colOff>444499</xdr:colOff>
+      <xdr:row>165</xdr:row>
+      <xdr:rowOff>79375</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>11</xdr:col>
+      <xdr:colOff>262016</xdr:colOff>
+      <xdr:row>181</xdr:row>
+      <xdr:rowOff>45655</xdr:rowOff>
+    </xdr:to>
+    <xdr:pic>
+      <xdr:nvPicPr>
+        <xdr:cNvPr id="21" name="Image 20"/>
         <xdr:cNvPicPr>
           <a:picLocks noChangeAspect="1"/>
         </xdr:cNvPicPr>
@@ -1266,8 +1342,96 @@
       </xdr:blipFill>
       <xdr:spPr>
         <a:xfrm>
-          <a:off x="11287125" y="20018376"/>
-          <a:ext cx="5913632" cy="3086367"/>
+          <a:off x="7040562" y="30392688"/>
+          <a:ext cx="4580017" cy="2911092"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+      </xdr:spPr>
+    </xdr:pic>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+  <xdr:twoCellAnchor editAs="oneCell">
+    <xdr:from>
+      <xdr:col>5</xdr:col>
+      <xdr:colOff>500062</xdr:colOff>
+      <xdr:row>184</xdr:row>
+      <xdr:rowOff>15875</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>15</xdr:col>
+      <xdr:colOff>91774</xdr:colOff>
+      <xdr:row>201</xdr:row>
+      <xdr:rowOff>119976</xdr:rowOff>
+    </xdr:to>
+    <xdr:pic>
+      <xdr:nvPicPr>
+        <xdr:cNvPr id="22" name="Image 21"/>
+        <xdr:cNvPicPr>
+          <a:picLocks noChangeAspect="1"/>
+        </xdr:cNvPicPr>
+      </xdr:nvPicPr>
+      <xdr:blipFill>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId18">
+          <a:extLst>
+            <a:ext uri="{28A0092B-C50C-407E-A947-70E740481C1C}">
+              <a14:useLocalDpi xmlns:a14="http://schemas.microsoft.com/office/drawing/2010/main" val="0"/>
+            </a:ext>
+          </a:extLst>
+        </a:blip>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </xdr:blipFill>
+      <xdr:spPr>
+        <a:xfrm>
+          <a:off x="7096125" y="33829625"/>
+          <a:ext cx="7529212" cy="3223539"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+      </xdr:spPr>
+    </xdr:pic>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+  <xdr:twoCellAnchor editAs="oneCell">
+    <xdr:from>
+      <xdr:col>5</xdr:col>
+      <xdr:colOff>484187</xdr:colOff>
+      <xdr:row>202</xdr:row>
+      <xdr:rowOff>79375</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>14</xdr:col>
+      <xdr:colOff>785812</xdr:colOff>
+      <xdr:row>225</xdr:row>
+      <xdr:rowOff>95249</xdr:rowOff>
+    </xdr:to>
+    <xdr:pic>
+      <xdr:nvPicPr>
+        <xdr:cNvPr id="23" name="Image 22"/>
+        <xdr:cNvPicPr>
+          <a:picLocks noChangeAspect="1"/>
+        </xdr:cNvPicPr>
+      </xdr:nvPicPr>
+      <xdr:blipFill>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId19">
+          <a:extLst>
+            <a:ext uri="{28A0092B-C50C-407E-A947-70E740481C1C}">
+              <a14:useLocalDpi xmlns:a14="http://schemas.microsoft.com/office/drawing/2010/main" val="0"/>
+            </a:ext>
+          </a:extLst>
+        </a:blip>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </xdr:blipFill>
+      <xdr:spPr>
+        <a:xfrm>
+          <a:off x="7080250" y="37195125"/>
+          <a:ext cx="7445375" cy="4254499"/>
         </a:xfrm>
         <a:prstGeom prst="rect">
           <a:avLst/>
@@ -1542,7 +1706,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:E232"/>
+  <dimension ref="A1:R232"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="52.6640625" bestFit="1" customWidth="1"/>
@@ -1550,6 +1714,7 @@
     <col min="3" max="3" width="12" bestFit="1" customWidth="1"/>
     <col min="4" max="4" width="10" bestFit="1" customWidth="1"/>
     <col min="5" max="5" width="11" bestFit="1" customWidth="1"/>
+    <col min="18" max="18" width="13.21875" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:5" ht="15" thickBot="1" x14ac:dyDescent="0.35">
@@ -1560,13 +1725,13 @@
         <v>0</v>
       </c>
       <c r="C1" s="5" t="s">
-        <v>42</v>
+        <v>34</v>
       </c>
       <c r="D1" s="5" t="s">
-        <v>43</v>
+        <v>35</v>
       </c>
       <c r="E1" s="14" t="s">
-        <v>44</v>
+        <v>36</v>
       </c>
     </row>
     <row r="2" spans="1:5" x14ac:dyDescent="0.3">
@@ -1580,10 +1745,10 @@
         <v>0</v>
       </c>
       <c r="D2" s="7" t="s">
-        <v>45</v>
+        <v>37</v>
       </c>
       <c r="E2" s="7" t="s">
-        <v>48</v>
+        <v>40</v>
       </c>
     </row>
     <row r="3" spans="1:5" x14ac:dyDescent="0.3">
@@ -1597,10 +1762,10 @@
         <v>0</v>
       </c>
       <c r="D3" s="2" t="s">
-        <v>49</v>
+        <v>41</v>
       </c>
       <c r="E3" s="2" t="s">
-        <v>47</v>
+        <v>39</v>
       </c>
     </row>
     <row r="4" spans="1:5" ht="15" thickBot="1" x14ac:dyDescent="0.35">
@@ -1614,10 +1779,10 @@
         <v>0</v>
       </c>
       <c r="D4" s="3" t="s">
-        <v>50</v>
+        <v>42</v>
       </c>
       <c r="E4" s="3" t="s">
-        <v>46</v>
+        <v>38</v>
       </c>
     </row>
     <row r="5" spans="1:5" x14ac:dyDescent="0.3">
@@ -1632,13 +1797,13 @@
         <v>0</v>
       </c>
       <c r="C23" s="5" t="s">
-        <v>42</v>
+        <v>34</v>
       </c>
       <c r="D23" s="5" t="s">
-        <v>43</v>
+        <v>35</v>
       </c>
       <c r="E23" s="14" t="s">
-        <v>44</v>
+        <v>36</v>
       </c>
     </row>
     <row r="24" spans="1:5" ht="15" thickBot="1" x14ac:dyDescent="0.35">
@@ -1649,13 +1814,13 @@
         <v>10</v>
       </c>
       <c r="C24" s="5" t="s">
-        <v>51</v>
+        <v>43</v>
       </c>
       <c r="D24" s="5" t="s">
-        <v>52</v>
+        <v>44</v>
       </c>
       <c r="E24" s="5" t="s">
-        <v>53</v>
+        <v>45</v>
       </c>
     </row>
     <row r="40" spans="1:5" ht="15" thickBot="1" x14ac:dyDescent="0.35"/>
@@ -1667,13 +1832,13 @@
         <v>0</v>
       </c>
       <c r="C41" s="5" t="s">
-        <v>42</v>
+        <v>34</v>
       </c>
       <c r="D41" s="5" t="s">
-        <v>43</v>
+        <v>35</v>
       </c>
       <c r="E41" s="14" t="s">
-        <v>44</v>
+        <v>36</v>
       </c>
     </row>
     <row r="42" spans="1:5" ht="15" thickBot="1" x14ac:dyDescent="0.35">
@@ -1684,13 +1849,13 @@
         <v>11</v>
       </c>
       <c r="C42" s="2" t="s">
-        <v>57</v>
+        <v>49</v>
       </c>
       <c r="D42" s="2" t="s">
-        <v>56</v>
+        <v>48</v>
       </c>
       <c r="E42" s="2" t="s">
-        <v>55</v>
+        <v>47</v>
       </c>
     </row>
     <row r="43" spans="1:5" ht="15" thickBot="1" x14ac:dyDescent="0.35">
@@ -1701,13 +1866,13 @@
         <v>12</v>
       </c>
       <c r="C43" s="3" t="s">
-        <v>58</v>
+        <v>50</v>
       </c>
       <c r="D43" s="3" t="s">
-        <v>59</v>
+        <v>51</v>
       </c>
       <c r="E43" s="3" t="s">
-        <v>54</v>
+        <v>46</v>
       </c>
     </row>
     <row r="71" spans="1:5" ht="15" thickBot="1" x14ac:dyDescent="0.35"/>
@@ -1719,13 +1884,13 @@
         <v>0</v>
       </c>
       <c r="C72" s="5" t="s">
-        <v>42</v>
+        <v>34</v>
       </c>
       <c r="D72" s="5" t="s">
-        <v>43</v>
+        <v>35</v>
       </c>
       <c r="E72" s="14" t="s">
-        <v>44</v>
+        <v>36</v>
       </c>
     </row>
     <row r="73" spans="1:5" ht="15" thickBot="1" x14ac:dyDescent="0.35">
@@ -1736,13 +1901,13 @@
         <v>15</v>
       </c>
       <c r="C73" s="3" t="s">
-        <v>62</v>
+        <v>54</v>
       </c>
       <c r="D73" s="3" t="s">
-        <v>61</v>
+        <v>53</v>
       </c>
       <c r="E73" s="3" t="s">
-        <v>60</v>
+        <v>52</v>
       </c>
     </row>
     <row r="74" spans="1:5" x14ac:dyDescent="0.3">
@@ -1758,18 +1923,18 @@
         <v>0</v>
       </c>
       <c r="C88" s="9" t="s">
-        <v>42</v>
+        <v>34</v>
       </c>
       <c r="D88" s="9" t="s">
-        <v>43</v>
+        <v>35</v>
       </c>
       <c r="E88" s="15" t="s">
-        <v>44</v>
+        <v>36</v>
       </c>
     </row>
     <row r="89" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A89" s="7" t="s">
-        <v>22</v>
+        <v>20</v>
       </c>
       <c r="B89" s="11" t="s">
         <v>17</v>
@@ -1778,44 +1943,44 @@
         <v>0</v>
       </c>
       <c r="D89" s="7" t="s">
-        <v>63</v>
+        <v>55</v>
       </c>
       <c r="E89" s="16" t="s">
-        <v>64</v>
+        <v>56</v>
       </c>
     </row>
     <row r="90" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A90" s="2" t="s">
-        <v>23</v>
+        <v>21</v>
       </c>
       <c r="B90" s="12" t="s">
         <v>18</v>
       </c>
       <c r="C90" s="2" t="s">
-        <v>65</v>
+        <v>57</v>
       </c>
       <c r="D90" s="2" t="s">
-        <v>66</v>
+        <v>58</v>
       </c>
       <c r="E90" s="17" t="s">
-        <v>67</v>
+        <v>59</v>
       </c>
     </row>
     <row r="91" spans="1:5" ht="15" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A91" s="3" t="s">
-        <v>24</v>
+        <v>22</v>
       </c>
       <c r="B91" s="13" t="s">
         <v>19</v>
       </c>
       <c r="C91" s="3" t="s">
-        <v>68</v>
+        <v>60</v>
       </c>
       <c r="D91" s="3" t="s">
-        <v>69</v>
+        <v>61</v>
       </c>
       <c r="E91" s="18" t="s">
-        <v>70</v>
+        <v>62</v>
       </c>
     </row>
     <row r="110" spans="1:5" ht="15" thickBot="1" x14ac:dyDescent="0.35"/>
@@ -1827,34 +1992,34 @@
         <v>0</v>
       </c>
       <c r="C111" s="5" t="s">
-        <v>42</v>
+        <v>34</v>
       </c>
       <c r="D111" s="5" t="s">
-        <v>43</v>
+        <v>35</v>
       </c>
       <c r="E111" s="14" t="s">
-        <v>44</v>
+        <v>36</v>
       </c>
     </row>
     <row r="112" spans="1:5" ht="15" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A112" s="5" t="s">
-        <v>71</v>
+        <v>63</v>
       </c>
       <c r="B112" s="5" t="s">
-        <v>25</v>
+        <v>23</v>
       </c>
       <c r="C112" s="19" t="s">
-        <v>72</v>
+        <v>64</v>
       </c>
       <c r="D112" s="19" t="s">
-        <v>73</v>
+        <v>65</v>
       </c>
       <c r="E112" s="20" t="s">
-        <v>74</v>
-      </c>
-    </row>
-    <row r="126" spans="1:5" ht="15" thickBot="1" x14ac:dyDescent="0.35"/>
-    <row r="127" spans="1:5" ht="15" thickBot="1" x14ac:dyDescent="0.35">
+        <v>66</v>
+      </c>
+    </row>
+    <row r="126" spans="1:18" ht="15" thickBot="1" x14ac:dyDescent="0.35"/>
+    <row r="127" spans="1:18" ht="15" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A127" s="6" t="s">
         <v>8</v>
       </c>
@@ -1862,114 +2027,239 @@
         <v>0</v>
       </c>
       <c r="C127" s="5" t="s">
-        <v>42</v>
+        <v>34</v>
       </c>
       <c r="D127" s="5" t="s">
-        <v>43</v>
+        <v>35</v>
       </c>
       <c r="E127" s="14" t="s">
-        <v>44</v>
-      </c>
-    </row>
-    <row r="128" spans="1:5" ht="15" thickBot="1" x14ac:dyDescent="0.35">
+        <v>36</v>
+      </c>
+    </row>
+    <row r="128" spans="1:18" ht="15" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A128" s="5" t="s">
-        <v>21</v>
+        <v>71</v>
       </c>
       <c r="B128" s="5" t="s">
-        <v>20</v>
-      </c>
-    </row>
-    <row r="133" spans="1:1" x14ac:dyDescent="0.3">
-      <c r="A133" t="s">
-        <v>36</v>
-      </c>
-    </row>
-    <row r="146" spans="1:2" ht="15" thickBot="1" x14ac:dyDescent="0.35"/>
-    <row r="147" spans="1:2" ht="15" thickBot="1" x14ac:dyDescent="0.35">
+        <v>67</v>
+      </c>
+      <c r="C128" s="19" t="s">
+        <v>68</v>
+      </c>
+      <c r="D128" s="19" t="s">
+        <v>69</v>
+      </c>
+      <c r="E128" s="20" t="s">
+        <v>70</v>
+      </c>
+      <c r="R128" t="s">
+        <v>72</v>
+      </c>
+    </row>
+    <row r="146" spans="1:5" ht="15" thickBot="1" x14ac:dyDescent="0.35"/>
+    <row r="147" spans="1:5" ht="15" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A147" s="6" t="s">
         <v>8</v>
       </c>
       <c r="B147" s="5" t="s">
         <v>0</v>
       </c>
-    </row>
-    <row r="148" spans="1:2" ht="15" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="C147" s="5" t="s">
+        <v>34</v>
+      </c>
+      <c r="D147" s="5" t="s">
+        <v>35</v>
+      </c>
+      <c r="E147" s="14" t="s">
+        <v>36</v>
+      </c>
+    </row>
+    <row r="148" spans="1:5" ht="15" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A148" s="5" t="s">
-        <v>26</v>
+        <v>24</v>
       </c>
       <c r="B148" s="5" t="s">
-        <v>27</v>
-      </c>
-    </row>
-    <row r="167" spans="1:2" ht="15" thickBot="1" x14ac:dyDescent="0.35"/>
-    <row r="168" spans="1:2" ht="15" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="A168" s="6" t="s">
-        <v>8</v>
+        <v>25</v>
+      </c>
+      <c r="C148" s="19" t="s">
+        <v>73</v>
+      </c>
+      <c r="D148" s="19" t="s">
+        <v>74</v>
+      </c>
+      <c r="E148" s="20" t="s">
+        <v>75</v>
+      </c>
+    </row>
+    <row r="167" spans="1:5" ht="15" thickBot="1" x14ac:dyDescent="0.35"/>
+    <row r="168" spans="1:5" ht="15" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="A168" s="8" t="s">
+        <v>7</v>
       </c>
       <c r="B168" s="5" t="s">
         <v>0</v>
       </c>
-    </row>
-    <row r="169" spans="1:2" ht="15" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="A169" s="5" t="s">
-        <v>30</v>
-      </c>
-      <c r="B169" s="5" t="s">
-        <v>28</v>
-      </c>
-    </row>
-    <row r="174" spans="1:2" x14ac:dyDescent="0.3">
-      <c r="A174" t="s">
-        <v>37</v>
-      </c>
-    </row>
-    <row r="184" spans="1:2" ht="15" thickBot="1" x14ac:dyDescent="0.35"/>
-    <row r="185" spans="1:2" ht="15" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="C168" s="5" t="s">
+        <v>34</v>
+      </c>
+      <c r="D168" s="5" t="s">
+        <v>35</v>
+      </c>
+      <c r="E168" s="14" t="s">
+        <v>36</v>
+      </c>
+    </row>
+    <row r="169" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A169" s="7" t="s">
+        <v>77</v>
+      </c>
+      <c r="B169" s="16" t="s">
+        <v>81</v>
+      </c>
+      <c r="C169" s="21">
+        <v>1</v>
+      </c>
+      <c r="D169" s="4">
+        <v>8</v>
+      </c>
+      <c r="E169" s="4" t="s">
+        <v>79</v>
+      </c>
+    </row>
+    <row r="170" spans="1:5" ht="15" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="A170" s="3" t="s">
+        <v>76</v>
+      </c>
+      <c r="B170" s="18" t="s">
+        <v>80</v>
+      </c>
+      <c r="C170" s="18">
+        <v>0</v>
+      </c>
+      <c r="D170" s="3">
+        <v>8</v>
+      </c>
+      <c r="E170" s="3" t="s">
+        <v>78</v>
+      </c>
+    </row>
+    <row r="184" spans="1:5" ht="15" thickBot="1" x14ac:dyDescent="0.35"/>
+    <row r="185" spans="1:5" ht="15" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A185" s="6" t="s">
         <v>8</v>
       </c>
       <c r="B185" s="5" t="s">
         <v>0</v>
       </c>
-    </row>
-    <row r="186" spans="1:2" ht="15" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="C185" s="5" t="s">
+        <v>34</v>
+      </c>
+      <c r="D185" s="5" t="s">
+        <v>35</v>
+      </c>
+      <c r="E185" s="14" t="s">
+        <v>36</v>
+      </c>
+    </row>
+    <row r="186" spans="1:5" ht="15" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A186" s="5" t="s">
-        <v>29</v>
+        <v>26</v>
       </c>
       <c r="B186" s="5" t="s">
-        <v>31</v>
-      </c>
-    </row>
-    <row r="205" spans="1:2" ht="15" thickBot="1" x14ac:dyDescent="0.35"/>
-    <row r="206" spans="1:2" ht="15" thickBot="1" x14ac:dyDescent="0.35">
+        <v>27</v>
+      </c>
+      <c r="C186" s="19" t="s">
+        <v>84</v>
+      </c>
+      <c r="D186" s="19" t="s">
+        <v>83</v>
+      </c>
+      <c r="E186" s="20" t="s">
+        <v>82</v>
+      </c>
+    </row>
+    <row r="205" spans="1:5" ht="15" thickBot="1" x14ac:dyDescent="0.35"/>
+    <row r="206" spans="1:5" ht="15" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A206" s="6" t="s">
         <v>8</v>
       </c>
-      <c r="B206" s="5" t="s">
+      <c r="B206" s="9" t="s">
         <v>0</v>
       </c>
-    </row>
-    <row r="207" spans="1:2" ht="15" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="A207" s="5" t="s">
-        <v>33</v>
-      </c>
-      <c r="B207" s="5" t="s">
+      <c r="C206" s="9" t="s">
+        <v>34</v>
+      </c>
+      <c r="D206" s="9" t="s">
+        <v>35</v>
+      </c>
+      <c r="E206" s="15" t="s">
+        <v>36</v>
+      </c>
+    </row>
+    <row r="207" spans="1:5" ht="15" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="A207" s="10" t="s">
+        <v>93</v>
+      </c>
+      <c r="B207" s="7" t="s">
+        <v>86</v>
+      </c>
+      <c r="C207" s="7">
+        <v>11</v>
+      </c>
+      <c r="D207" s="7">
+        <v>31</v>
+      </c>
+      <c r="E207" s="7" t="s">
+        <v>85</v>
+      </c>
+    </row>
+    <row r="208" spans="1:5" ht="15" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="A208" s="10" t="s">
+        <v>91</v>
+      </c>
+      <c r="B208" s="2" t="s">
+        <v>87</v>
+      </c>
+      <c r="C208" s="2">
+        <v>1</v>
+      </c>
+      <c r="D208" s="2">
+        <v>9</v>
+      </c>
+      <c r="E208" s="2" t="s">
+        <v>88</v>
+      </c>
+    </row>
+    <row r="209" spans="1:5" ht="15" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="A209" s="10" t="s">
+        <v>92</v>
+      </c>
+      <c r="B209" s="3" t="s">
+        <v>89</v>
+      </c>
+      <c r="C209" s="3">
+        <v>2</v>
+      </c>
+      <c r="D209" s="3">
+        <v>31</v>
+      </c>
+      <c r="E209" s="3" t="s">
+        <v>90</v>
+      </c>
+    </row>
+    <row r="212" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A212" s="22" t="s">
+        <v>30</v>
+      </c>
+    </row>
+    <row r="213" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A213" s="22" t="s">
+        <v>31</v>
+      </c>
+    </row>
+    <row r="214" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A214" s="22" t="s">
         <v>32</v>
-      </c>
-    </row>
-    <row r="212" spans="1:1" x14ac:dyDescent="0.3">
-      <c r="A212" t="s">
-        <v>38</v>
-      </c>
-    </row>
-    <row r="213" spans="1:1" x14ac:dyDescent="0.3">
-      <c r="A213" t="s">
-        <v>39</v>
-      </c>
-    </row>
-    <row r="214" spans="1:1" x14ac:dyDescent="0.3">
-      <c r="A214" t="s">
-        <v>40</v>
       </c>
     </row>
     <row r="226" spans="1:2" ht="15" thickBot="1" x14ac:dyDescent="0.35"/>
@@ -1983,15 +2273,15 @@
     </row>
     <row r="228" spans="1:2" ht="15" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A228" s="5" t="s">
-        <v>35</v>
+        <v>29</v>
       </c>
       <c r="B228" s="5" t="s">
-        <v>34</v>
+        <v>28</v>
       </c>
     </row>
     <row r="232" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A232" t="s">
-        <v>41</v>
+        <v>33</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
29/04/25 : rajout des seuils 0-2m et vérif intégrales des metriques
</commit_message>
<xml_diff>
--- a/Graphiques_&_ECARTYPES_Metriques_AD.xlsx
+++ b/Graphiques_&_ECARTYPES_Metriques_AD.xlsx
@@ -9,11 +9,12 @@
     </mc:Choice>
   </mc:AlternateContent>
   <bookViews>
-    <workbookView xWindow="0" yWindow="0" windowWidth="23040" windowHeight="9192"/>
+    <workbookView xWindow="0" yWindow="0" windowWidth="23040" windowHeight="9192" firstSheet="1" activeTab="1"/>
   </bookViews>
   <sheets>
     <sheet name="Graphiques_variances_metriques" sheetId="1" r:id="rId1"/>
-    <sheet name="Informations_metriques" sheetId="2" r:id="rId2"/>
+    <sheet name="Matrices_corrélations" sheetId="3" r:id="rId2"/>
+    <sheet name="Informations_metriques" sheetId="2" r:id="rId3"/>
   </sheets>
   <calcPr calcId="162913" refMode="R1C1"/>
   <extLst>
@@ -25,7 +26,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="231" uniqueCount="94">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="259" uniqueCount="122">
   <si>
     <t>Ecart-type</t>
   </si>
@@ -307,6 +308,1274 @@
   </si>
   <si>
     <t>Metriques_DiversiteBM_Placette_AD : échelle placette</t>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>BMS</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve"> placette corrélé avec </t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>BMP</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve"> placette understory à hauteur de 0,66</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>BMS</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve"> placette corrélé avec </t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>BMtot</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve"> placette à hauteur de 0,68</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>BMS</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve"> placette corrélé avec </t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>NBespBM</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve"> placette à hauteur de 0,69</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>BMS</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve"> placette corrélé avec </t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>NBespBM</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve"> understory placette à hauteur de 0,64</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <t xml:space="preserve">Volume de </t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>BMP+BMD</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve"> corrélé fortement avec Volume de </t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>BMP</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve"> placette à hauteur de 0,91</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <t xml:space="preserve">Volume de </t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>BMP+BMD</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve"> corrélé fortement avec </t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>BMtot</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve"> placette à hauteur de 0,92</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <t xml:space="preserve">Volume de </t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>BMP+BMD</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve"> corrélé avec </t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>NBespBM</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve"> placette à hauteur de 0,6</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>Bmtot</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve"> corrélé fortement avec Volume de </t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>BMP+BMD</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve"> à hauteur de 0,92</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>Bmtot</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve"> corrélé fortement avec Volume de </t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>BMD</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve"> placette à hauteur de 0,82</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>Bmtot</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve"> corrélé avec </t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>NBespBM</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve"> understory placette à hauteur de 0,73</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>Bmtot</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve"> corrélé avec </t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>BMS</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve"> placette à hauteur de 0,68</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>Bmtot</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve"> corrélé avec </t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>NBespBM</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve"> placette à hauteur de 0,76</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <t xml:space="preserve">Volume </t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>BMD</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve"> placette corrélé fortement avec Volume </t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>BMD+BMP</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve"> à hauteur de 0,91</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <t>Volume</t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve"> BMD</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve"> placette corrélé fortement avec </t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>Bmtot</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve"> à hauteur de 0,82</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve">NBespBM </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve">placette corrélé fortement avec </t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>NBespBM</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve"> understory placette à hauteur de 0,99</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>NBespBM</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve"> placette corrélé avec </t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>Bmtot</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve"> à hauteur de 0,76</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>NBespBM</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve"> placette corrélé avec Volume de </t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>BMP+BMD</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve"> à hauteur de 0,6</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>NBespBM</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve"> placette corrélé avec </t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>BMS</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve"> placette à hauteur de 0,69</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>NBespBM</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve"> understory placette corrélé fortement avec </t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>NBespBM</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve"> à hauteur de 0,99</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>NBespBM</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve"> understory placette corrélé avec </t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>BMS</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve"> placette à hauteur de 0,64</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>NBespBM</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve"> understory placette corrélé avec </t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>Bmtot</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve"> à hauteur de 0,73</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <t>Volume</t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve"> BMP </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve">canopy corrélé fortement avec Volume </t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>BMP</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve"> placette pondéré à hauteur de 0,9</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <t xml:space="preserve">Volume </t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>BMP</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve"> placette pondéré corrélé fortement avec Volume </t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>BMP</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve"> canopy  à hauteur de 0,9</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <t xml:space="preserve">Volume </t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>BMP</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve"> below-canopy corrélé avec Volume </t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>BMP</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve"> understory à hauteur de 0,72</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <t xml:space="preserve">Volume </t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>BMP</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve"> understory corrélé avec </t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>BMS</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve"> placette à hauteur de 0,66</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <t xml:space="preserve">Volume </t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>BMP</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve"> understory corrélé avec Volume </t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>BMP</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve"> below-canopy à hauteur de 0,72</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <t xml:space="preserve">Volume </t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>BMP</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve"> lower-canopy corrélé fortement avec Volume </t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>BMP</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve"> arbre à hauteur de 0,93</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <t xml:space="preserve">Volume </t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>BMP</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve"> arbre corrélé fortement avec Volume </t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>BMP</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve"> lower-canopy à hauteur de 0,93</t>
+    </r>
   </si>
 </sst>
 </file>
@@ -330,7 +1599,7 @@
       <scheme val="minor"/>
     </font>
   </fonts>
-  <fills count="14">
+  <fills count="15">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -409,6 +1678,12 @@
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFEC4A46"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
   </fills>
   <borders count="20">
     <border>
@@ -667,7 +1942,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="75">
+  <cellXfs count="76">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyBorder="1"/>
@@ -751,12 +2026,18 @@
     <xf numFmtId="0" fontId="0" fillId="10" borderId="12" xfId="0" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="10" borderId="3" xfId="0" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="10" borderId="13" xfId="0" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="14" borderId="0" xfId="0" applyFill="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
   <dxfs count="0"/>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium2" defaultPivotStyle="PivotStyleLight16"/>
+  <colors>
+    <mruColors>
+      <color rgb="FFEC4A46"/>
+    </mruColors>
+  </colors>
   <extLst>
     <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{EB79DEF2-80B8-43e5-95BD-54CBDDF9020C}">
       <x14:slicerStyles defaultSlicerStyle="SlicerStyleLight1"/>
@@ -1609,6 +2890,55 @@
 </xdr:wsDr>
 </file>
 
+<file path=xl/drawings/drawing2.xml><?xml version="1.0" encoding="utf-8"?>
+<xdr:wsDr xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+  <xdr:twoCellAnchor editAs="oneCell">
+    <xdr:from>
+      <xdr:col>1</xdr:col>
+      <xdr:colOff>83820</xdr:colOff>
+      <xdr:row>0</xdr:row>
+      <xdr:rowOff>53340</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>10</xdr:col>
+      <xdr:colOff>723900</xdr:colOff>
+      <xdr:row>42</xdr:row>
+      <xdr:rowOff>144780</xdr:rowOff>
+    </xdr:to>
+    <xdr:pic>
+      <xdr:nvPicPr>
+        <xdr:cNvPr id="2" name="Image 1"/>
+        <xdr:cNvPicPr>
+          <a:picLocks noChangeAspect="1"/>
+        </xdr:cNvPicPr>
+      </xdr:nvPicPr>
+      <xdr:blipFill>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId1" cstate="print">
+          <a:extLst>
+            <a:ext uri="{28A0092B-C50C-407E-A947-70E740481C1C}">
+              <a14:useLocalDpi xmlns:a14="http://schemas.microsoft.com/office/drawing/2010/main" val="0"/>
+            </a:ext>
+          </a:extLst>
+        </a:blip>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </xdr:blipFill>
+      <xdr:spPr>
+        <a:xfrm>
+          <a:off x="5326380" y="53340"/>
+          <a:ext cx="7772400" cy="7772400"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+      </xdr:spPr>
+    </xdr:pic>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+</xdr:wsDr>
+</file>
+
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
 <a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Thème Office">
   <a:themeElements>
@@ -2459,6 +3789,161 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+  <dimension ref="A2:A40"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <cols>
+    <col min="1" max="1" width="76.44140625" bestFit="1" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="2" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="A2" t="s">
+        <v>94</v>
+      </c>
+    </row>
+    <row r="3" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="A3" t="s">
+        <v>95</v>
+      </c>
+    </row>
+    <row r="4" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="A4" t="s">
+        <v>96</v>
+      </c>
+    </row>
+    <row r="5" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="A5" t="s">
+        <v>97</v>
+      </c>
+    </row>
+    <row r="7" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="A7" t="s">
+        <v>99</v>
+      </c>
+    </row>
+    <row r="8" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="A8" t="s">
+        <v>98</v>
+      </c>
+    </row>
+    <row r="9" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="A9" t="s">
+        <v>100</v>
+      </c>
+    </row>
+    <row r="11" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="A11" t="s">
+        <v>102</v>
+      </c>
+    </row>
+    <row r="12" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="A12" t="s">
+        <v>101</v>
+      </c>
+    </row>
+    <row r="13" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="A13" t="s">
+        <v>104</v>
+      </c>
+    </row>
+    <row r="14" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="A14" t="s">
+        <v>105</v>
+      </c>
+    </row>
+    <row r="15" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="A15" t="s">
+        <v>103</v>
+      </c>
+    </row>
+    <row r="17" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="A17" t="s">
+        <v>107</v>
+      </c>
+    </row>
+    <row r="18" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="A18" t="s">
+        <v>106</v>
+      </c>
+    </row>
+    <row r="20" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="A20" t="s">
+        <v>108</v>
+      </c>
+    </row>
+    <row r="21" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="A21" t="s">
+        <v>109</v>
+      </c>
+    </row>
+    <row r="22" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="A22" t="s">
+        <v>110</v>
+      </c>
+    </row>
+    <row r="23" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="A23" t="s">
+        <v>111</v>
+      </c>
+    </row>
+    <row r="25" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="A25" t="s">
+        <v>114</v>
+      </c>
+    </row>
+    <row r="26" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="A26" t="s">
+        <v>113</v>
+      </c>
+    </row>
+    <row r="27" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="A27" t="s">
+        <v>112</v>
+      </c>
+    </row>
+    <row r="29" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="A29" t="s">
+        <v>115</v>
+      </c>
+    </row>
+    <row r="31" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="A31" t="s">
+        <v>116</v>
+      </c>
+    </row>
+    <row r="33" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="A33" t="s">
+        <v>117</v>
+      </c>
+    </row>
+    <row r="35" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="A35" t="s">
+        <v>119</v>
+      </c>
+    </row>
+    <row r="36" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="A36" s="75" t="s">
+        <v>118</v>
+      </c>
+    </row>
+    <row r="38" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="A38" s="75" t="s">
+        <v>120</v>
+      </c>
+    </row>
+    <row r="40" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="A40" s="75" t="s">
+        <v>121</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup paperSize="9" orientation="portrait" r:id="rId1"/>
+  <drawing r:id="rId2"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
   <dimension ref="A1:E20"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>

</xml_diff>

<commit_message>
30-04-25 : regarder le jeu de données entomo début
</commit_message>
<xml_diff>
--- a/Graphiques_&_ECARTYPES_Metriques_AD.xlsx
+++ b/Graphiques_&_ECARTYPES_Metriques_AD.xlsx
@@ -9,12 +9,12 @@
     </mc:Choice>
   </mc:AlternateContent>
   <bookViews>
-    <workbookView xWindow="0" yWindow="0" windowWidth="23040" windowHeight="9192" firstSheet="1" activeTab="1"/>
+    <workbookView xWindow="0" yWindow="0" windowWidth="23040" windowHeight="9192" activeTab="2"/>
   </bookViews>
   <sheets>
     <sheet name="Graphiques_variances_metriques" sheetId="1" r:id="rId1"/>
-    <sheet name="Matrices_corrélations" sheetId="3" r:id="rId2"/>
-    <sheet name="Informations_metriques" sheetId="2" r:id="rId3"/>
+    <sheet name="Informations_metriques" sheetId="2" r:id="rId2"/>
+    <sheet name="Matrices_corrélations" sheetId="3" r:id="rId3"/>
   </sheets>
   <calcPr calcId="162913" refMode="R1C1"/>
   <extLst>
@@ -3789,161 +3789,6 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A2:A40"/>
-  <sheetFormatPr baseColWidth="10" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
-  <cols>
-    <col min="1" max="1" width="76.44140625" bestFit="1" customWidth="1"/>
-  </cols>
-  <sheetData>
-    <row r="2" spans="1:1" x14ac:dyDescent="0.3">
-      <c r="A2" t="s">
-        <v>94</v>
-      </c>
-    </row>
-    <row r="3" spans="1:1" x14ac:dyDescent="0.3">
-      <c r="A3" t="s">
-        <v>95</v>
-      </c>
-    </row>
-    <row r="4" spans="1:1" x14ac:dyDescent="0.3">
-      <c r="A4" t="s">
-        <v>96</v>
-      </c>
-    </row>
-    <row r="5" spans="1:1" x14ac:dyDescent="0.3">
-      <c r="A5" t="s">
-        <v>97</v>
-      </c>
-    </row>
-    <row r="7" spans="1:1" x14ac:dyDescent="0.3">
-      <c r="A7" t="s">
-        <v>99</v>
-      </c>
-    </row>
-    <row r="8" spans="1:1" x14ac:dyDescent="0.3">
-      <c r="A8" t="s">
-        <v>98</v>
-      </c>
-    </row>
-    <row r="9" spans="1:1" x14ac:dyDescent="0.3">
-      <c r="A9" t="s">
-        <v>100</v>
-      </c>
-    </row>
-    <row r="11" spans="1:1" x14ac:dyDescent="0.3">
-      <c r="A11" t="s">
-        <v>102</v>
-      </c>
-    </row>
-    <row r="12" spans="1:1" x14ac:dyDescent="0.3">
-      <c r="A12" t="s">
-        <v>101</v>
-      </c>
-    </row>
-    <row r="13" spans="1:1" x14ac:dyDescent="0.3">
-      <c r="A13" t="s">
-        <v>104</v>
-      </c>
-    </row>
-    <row r="14" spans="1:1" x14ac:dyDescent="0.3">
-      <c r="A14" t="s">
-        <v>105</v>
-      </c>
-    </row>
-    <row r="15" spans="1:1" x14ac:dyDescent="0.3">
-      <c r="A15" t="s">
-        <v>103</v>
-      </c>
-    </row>
-    <row r="17" spans="1:1" x14ac:dyDescent="0.3">
-      <c r="A17" t="s">
-        <v>107</v>
-      </c>
-    </row>
-    <row r="18" spans="1:1" x14ac:dyDescent="0.3">
-      <c r="A18" t="s">
-        <v>106</v>
-      </c>
-    </row>
-    <row r="20" spans="1:1" x14ac:dyDescent="0.3">
-      <c r="A20" t="s">
-        <v>108</v>
-      </c>
-    </row>
-    <row r="21" spans="1:1" x14ac:dyDescent="0.3">
-      <c r="A21" t="s">
-        <v>109</v>
-      </c>
-    </row>
-    <row r="22" spans="1:1" x14ac:dyDescent="0.3">
-      <c r="A22" t="s">
-        <v>110</v>
-      </c>
-    </row>
-    <row r="23" spans="1:1" x14ac:dyDescent="0.3">
-      <c r="A23" t="s">
-        <v>111</v>
-      </c>
-    </row>
-    <row r="25" spans="1:1" x14ac:dyDescent="0.3">
-      <c r="A25" t="s">
-        <v>114</v>
-      </c>
-    </row>
-    <row r="26" spans="1:1" x14ac:dyDescent="0.3">
-      <c r="A26" t="s">
-        <v>113</v>
-      </c>
-    </row>
-    <row r="27" spans="1:1" x14ac:dyDescent="0.3">
-      <c r="A27" t="s">
-        <v>112</v>
-      </c>
-    </row>
-    <row r="29" spans="1:1" x14ac:dyDescent="0.3">
-      <c r="A29" t="s">
-        <v>115</v>
-      </c>
-    </row>
-    <row r="31" spans="1:1" x14ac:dyDescent="0.3">
-      <c r="A31" t="s">
-        <v>116</v>
-      </c>
-    </row>
-    <row r="33" spans="1:1" x14ac:dyDescent="0.3">
-      <c r="A33" t="s">
-        <v>117</v>
-      </c>
-    </row>
-    <row r="35" spans="1:1" x14ac:dyDescent="0.3">
-      <c r="A35" t="s">
-        <v>119</v>
-      </c>
-    </row>
-    <row r="36" spans="1:1" x14ac:dyDescent="0.3">
-      <c r="A36" s="75" t="s">
-        <v>118</v>
-      </c>
-    </row>
-    <row r="38" spans="1:1" x14ac:dyDescent="0.3">
-      <c r="A38" s="75" t="s">
-        <v>120</v>
-      </c>
-    </row>
-    <row r="40" spans="1:1" x14ac:dyDescent="0.3">
-      <c r="A40" s="75" t="s">
-        <v>121</v>
-      </c>
-    </row>
-  </sheetData>
-  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <pageSetup paperSize="9" orientation="portrait" r:id="rId1"/>
-  <drawing r:id="rId2"/>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
   <dimension ref="A1:E20"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
@@ -4297,4 +4142,159 @@
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup paperSize="9" orientation="portrait" r:id="rId1"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+  <dimension ref="A2:A40"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <cols>
+    <col min="1" max="1" width="76.44140625" bestFit="1" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="2" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="A2" t="s">
+        <v>94</v>
+      </c>
+    </row>
+    <row r="3" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="A3" t="s">
+        <v>95</v>
+      </c>
+    </row>
+    <row r="4" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="A4" t="s">
+        <v>96</v>
+      </c>
+    </row>
+    <row r="5" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="A5" t="s">
+        <v>97</v>
+      </c>
+    </row>
+    <row r="7" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="A7" t="s">
+        <v>99</v>
+      </c>
+    </row>
+    <row r="8" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="A8" t="s">
+        <v>98</v>
+      </c>
+    </row>
+    <row r="9" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="A9" t="s">
+        <v>100</v>
+      </c>
+    </row>
+    <row r="11" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="A11" t="s">
+        <v>102</v>
+      </c>
+    </row>
+    <row r="12" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="A12" t="s">
+        <v>101</v>
+      </c>
+    </row>
+    <row r="13" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="A13" t="s">
+        <v>104</v>
+      </c>
+    </row>
+    <row r="14" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="A14" t="s">
+        <v>105</v>
+      </c>
+    </row>
+    <row r="15" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="A15" t="s">
+        <v>103</v>
+      </c>
+    </row>
+    <row r="17" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="A17" t="s">
+        <v>107</v>
+      </c>
+    </row>
+    <row r="18" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="A18" t="s">
+        <v>106</v>
+      </c>
+    </row>
+    <row r="20" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="A20" t="s">
+        <v>108</v>
+      </c>
+    </row>
+    <row r="21" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="A21" t="s">
+        <v>109</v>
+      </c>
+    </row>
+    <row r="22" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="A22" t="s">
+        <v>110</v>
+      </c>
+    </row>
+    <row r="23" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="A23" t="s">
+        <v>111</v>
+      </c>
+    </row>
+    <row r="25" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="A25" t="s">
+        <v>114</v>
+      </c>
+    </row>
+    <row r="26" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="A26" t="s">
+        <v>113</v>
+      </c>
+    </row>
+    <row r="27" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="A27" t="s">
+        <v>112</v>
+      </c>
+    </row>
+    <row r="29" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="A29" t="s">
+        <v>115</v>
+      </c>
+    </row>
+    <row r="31" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="A31" t="s">
+        <v>116</v>
+      </c>
+    </row>
+    <row r="33" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="A33" t="s">
+        <v>117</v>
+      </c>
+    </row>
+    <row r="35" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="A35" t="s">
+        <v>119</v>
+      </c>
+    </row>
+    <row r="36" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="A36" s="75" t="s">
+        <v>118</v>
+      </c>
+    </row>
+    <row r="38" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="A38" s="75" t="s">
+        <v>120</v>
+      </c>
+    </row>
+    <row r="40" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="A40" s="75" t="s">
+        <v>121</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup paperSize="9" orientation="portrait" r:id="rId1"/>
+  <drawing r:id="rId2"/>
+</worksheet>
 </file>
</xml_diff>

<commit_message>
20/05 : avancée dans analyses
</commit_message>
<xml_diff>
--- a/Graphiques_&_ECARTYPES_Metriques_AD.xlsx
+++ b/Graphiques_&_ECARTYPES_Metriques_AD.xlsx
@@ -9,7 +9,7 @@
     </mc:Choice>
   </mc:AlternateContent>
   <bookViews>
-    <workbookView xWindow="0" yWindow="0" windowWidth="23040" windowHeight="9192" activeTab="2"/>
+    <workbookView xWindow="0" yWindow="0" windowWidth="23040" windowHeight="9192"/>
   </bookViews>
   <sheets>
     <sheet name="Graphiques_variances_metriques" sheetId="1" r:id="rId1"/>
@@ -26,7 +26,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="259" uniqueCount="122">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="259" uniqueCount="128">
   <si>
     <t>Ecart-type</t>
   </si>
@@ -1576,6 +1576,24 @@
       </rPr>
       <t xml:space="preserve"> lower-canopy à hauteur de 0,93</t>
     </r>
+  </si>
+  <si>
+    <t>6.293047</t>
+  </si>
+  <si>
+    <t>22.14602</t>
+  </si>
+  <si>
+    <t>0.3290758</t>
+  </si>
+  <si>
+    <t>85.84921</t>
+  </si>
+  <si>
+    <t>34.91436</t>
+  </si>
+  <si>
+    <t>9.306923</t>
   </si>
 </sst>
 </file>
@@ -3342,7 +3360,7 @@
         <v>13</v>
       </c>
       <c r="B42" s="5" t="s">
-        <v>11</v>
+        <v>122</v>
       </c>
       <c r="C42" s="2" t="s">
         <v>49</v>
@@ -3351,7 +3369,7 @@
         <v>48</v>
       </c>
       <c r="E42" s="2" t="s">
-        <v>47</v>
+        <v>127</v>
       </c>
     </row>
     <row r="43" spans="1:5" ht="15" thickBot="1" x14ac:dyDescent="0.35">
@@ -3359,16 +3377,16 @@
         <v>14</v>
       </c>
       <c r="B43" s="5" t="s">
-        <v>12</v>
+        <v>123</v>
       </c>
       <c r="C43" s="3" t="s">
-        <v>50</v>
+        <v>124</v>
       </c>
       <c r="D43" s="3" t="s">
-        <v>51</v>
+        <v>125</v>
       </c>
       <c r="E43" s="3" t="s">
-        <v>46</v>
+        <v>126</v>
       </c>
     </row>
     <row r="71" spans="1:5" ht="15" thickBot="1" x14ac:dyDescent="0.35"/>

</xml_diff>

<commit_message>
07/07/25 : démarrage des glmm pour les différents relevées + essaie de continuer pour nestedness et turnover
</commit_message>
<xml_diff>
--- a/Graphiques_&_ECARTYPES_Metriques_AD.xlsx
+++ b/Graphiques_&_ECARTYPES_Metriques_AD.xlsx
@@ -26,7 +26,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="259" uniqueCount="128">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="259" uniqueCount="151">
   <si>
     <t>Ecart-type</t>
   </si>
@@ -1578,22 +1578,91 @@
     </r>
   </si>
   <si>
-    <t>6.293047</t>
-  </si>
-  <si>
-    <t>22.14602</t>
-  </si>
-  <si>
-    <t>0.3290758</t>
-  </si>
-  <si>
-    <t>85.84921</t>
-  </si>
-  <si>
-    <t>34.91436</t>
-  </si>
-  <si>
-    <t>9.306923</t>
+    <t>26.81507</t>
+  </si>
+  <si>
+    <t>29.56522</t>
+  </si>
+  <si>
+    <t>1.573265</t>
+  </si>
+  <si>
+    <t>0.01388889</t>
+  </si>
+  <si>
+    <t>6.111111</t>
+  </si>
+  <si>
+    <t>2.326736</t>
+  </si>
+  <si>
+    <t>5.536517</t>
+  </si>
+  <si>
+    <t>0.08226915</t>
+  </si>
+  <si>
+    <t>21.46235</t>
+  </si>
+  <si>
+    <t>8.72861</t>
+  </si>
+  <si>
+    <t>2.461241</t>
+  </si>
+  <si>
+    <t>8.048099</t>
+  </si>
+  <si>
+    <t>1.995315</t>
+  </si>
+  <si>
+    <t>12.45654</t>
+  </si>
+  <si>
+    <t>0.1847171</t>
+  </si>
+  <si>
+    <t>54.47871</t>
+  </si>
+  <si>
+    <t>8.312384</t>
+  </si>
+  <si>
+    <t>12.52651</t>
+  </si>
+  <si>
+    <t>0.5737986</t>
+  </si>
+  <si>
+    <t>55.85249</t>
+  </si>
+  <si>
+    <t>10.3077</t>
+  </si>
+  <si>
+    <t>36.64801</t>
+  </si>
+  <si>
+    <t>8.608548</t>
+  </si>
+  <si>
+    <t>159.0089</t>
+  </si>
+  <si>
+    <t>43.85607</t>
+  </si>
+  <si>
+    <t>13.90818</t>
+  </si>
+  <si>
+    <t>1.597314</t>
+  </si>
+  <si>
+    <t>64.96255</t>
+  </si>
+  <si>
+    <t>17.04099</t>
   </si>
 </sst>
 </file>
@@ -2159,50 +2228,6 @@
   </xdr:twoCellAnchor>
   <xdr:twoCellAnchor editAs="oneCell">
     <xdr:from>
-      <xdr:col>5</xdr:col>
-      <xdr:colOff>117793</xdr:colOff>
-      <xdr:row>70</xdr:row>
-      <xdr:rowOff>14922</xdr:rowOff>
-    </xdr:from>
-    <xdr:to>
-      <xdr:col>10</xdr:col>
-      <xdr:colOff>684288</xdr:colOff>
-      <xdr:row>85</xdr:row>
-      <xdr:rowOff>159954</xdr:rowOff>
-    </xdr:to>
-    <xdr:pic>
-      <xdr:nvPicPr>
-        <xdr:cNvPr id="6" name="Image 5"/>
-        <xdr:cNvPicPr>
-          <a:picLocks noChangeAspect="1"/>
-        </xdr:cNvPicPr>
-      </xdr:nvPicPr>
-      <xdr:blipFill>
-        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId3">
-          <a:extLst>
-            <a:ext uri="{28A0092B-C50C-407E-A947-70E740481C1C}">
-              <a14:useLocalDpi xmlns:a14="http://schemas.microsoft.com/office/drawing/2010/main" val="0"/>
-            </a:ext>
-          </a:extLst>
-        </a:blip>
-        <a:stretch>
-          <a:fillRect/>
-        </a:stretch>
-      </xdr:blipFill>
-      <xdr:spPr>
-        <a:xfrm>
-          <a:off x="6483668" y="12865735"/>
-          <a:ext cx="4535245" cy="2907282"/>
-        </a:xfrm>
-        <a:prstGeom prst="rect">
-          <a:avLst/>
-        </a:prstGeom>
-      </xdr:spPr>
-    </xdr:pic>
-    <xdr:clientData/>
-  </xdr:twoCellAnchor>
-  <xdr:twoCellAnchor editAs="oneCell">
-    <xdr:from>
       <xdr:col>26</xdr:col>
       <xdr:colOff>713152</xdr:colOff>
       <xdr:row>86</xdr:row>
@@ -2222,7 +2247,7 @@
         </xdr:cNvPicPr>
       </xdr:nvPicPr>
       <xdr:blipFill>
-        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId4">
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId3">
           <a:extLst>
             <a:ext uri="{28A0092B-C50C-407E-A947-70E740481C1C}">
               <a14:useLocalDpi xmlns:a14="http://schemas.microsoft.com/office/drawing/2010/main" val="0"/>
@@ -2266,7 +2291,7 @@
         </xdr:cNvPicPr>
       </xdr:nvPicPr>
       <xdr:blipFill>
-        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId5">
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId4">
           <a:extLst>
             <a:ext uri="{28A0092B-C50C-407E-A947-70E740481C1C}">
               <a14:useLocalDpi xmlns:a14="http://schemas.microsoft.com/office/drawing/2010/main" val="0"/>
@@ -2281,50 +2306,6 @@
         <a:xfrm>
           <a:off x="14928534" y="15804515"/>
           <a:ext cx="9073983" cy="4070703"/>
-        </a:xfrm>
-        <a:prstGeom prst="rect">
-          <a:avLst/>
-        </a:prstGeom>
-      </xdr:spPr>
-    </xdr:pic>
-    <xdr:clientData/>
-  </xdr:twoCellAnchor>
-  <xdr:twoCellAnchor editAs="oneCell">
-    <xdr:from>
-      <xdr:col>5</xdr:col>
-      <xdr:colOff>111125</xdr:colOff>
-      <xdr:row>108</xdr:row>
-      <xdr:rowOff>119062</xdr:rowOff>
-    </xdr:from>
-    <xdr:to>
-      <xdr:col>10</xdr:col>
-      <xdr:colOff>677620</xdr:colOff>
-      <xdr:row>124</xdr:row>
-      <xdr:rowOff>81215</xdr:rowOff>
-    </xdr:to>
-    <xdr:pic>
-      <xdr:nvPicPr>
-        <xdr:cNvPr id="10" name="Image 9"/>
-        <xdr:cNvPicPr>
-          <a:picLocks noChangeAspect="1"/>
-        </xdr:cNvPicPr>
-      </xdr:nvPicPr>
-      <xdr:blipFill>
-        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId6">
-          <a:extLst>
-            <a:ext uri="{28A0092B-C50C-407E-A947-70E740481C1C}">
-              <a14:useLocalDpi xmlns:a14="http://schemas.microsoft.com/office/drawing/2010/main" val="0"/>
-            </a:ext>
-          </a:extLst>
-        </a:blip>
-        <a:stretch>
-          <a:fillRect/>
-        </a:stretch>
-      </xdr:blipFill>
-      <xdr:spPr>
-        <a:xfrm>
-          <a:off x="6707188" y="19954875"/>
-          <a:ext cx="4535245" cy="2906965"/>
         </a:xfrm>
         <a:prstGeom prst="rect">
           <a:avLst/>
@@ -2354,7 +2335,7 @@
         </xdr:cNvPicPr>
       </xdr:nvPicPr>
       <xdr:blipFill>
-        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId7">
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId5">
           <a:extLst>
             <a:ext uri="{28A0092B-C50C-407E-A947-70E740481C1C}">
               <a14:useLocalDpi xmlns:a14="http://schemas.microsoft.com/office/drawing/2010/main" val="0"/>
@@ -2398,7 +2379,7 @@
         </xdr:cNvPicPr>
       </xdr:nvPicPr>
       <xdr:blipFill>
-        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId8">
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId6">
           <a:extLst>
             <a:ext uri="{28A0092B-C50C-407E-A947-70E740481C1C}">
               <a14:useLocalDpi xmlns:a14="http://schemas.microsoft.com/office/drawing/2010/main" val="0"/>
@@ -2442,7 +2423,7 @@
         </xdr:cNvPicPr>
       </xdr:nvPicPr>
       <xdr:blipFill>
-        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId9">
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId7">
           <a:extLst>
             <a:ext uri="{28A0092B-C50C-407E-A947-70E740481C1C}">
               <a14:useLocalDpi xmlns:a14="http://schemas.microsoft.com/office/drawing/2010/main" val="0"/>
@@ -2486,7 +2467,7 @@
         </xdr:cNvPicPr>
       </xdr:nvPicPr>
       <xdr:blipFill>
-        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId10">
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId8">
           <a:extLst>
             <a:ext uri="{28A0092B-C50C-407E-A947-70E740481C1C}">
               <a14:useLocalDpi xmlns:a14="http://schemas.microsoft.com/office/drawing/2010/main" val="0"/>
@@ -2501,226 +2482,6 @@
         <a:xfrm>
           <a:off x="11128375" y="4048126"/>
           <a:ext cx="4587638" cy="2911092"/>
-        </a:xfrm>
-        <a:prstGeom prst="rect">
-          <a:avLst/>
-        </a:prstGeom>
-      </xdr:spPr>
-    </xdr:pic>
-    <xdr:clientData/>
-  </xdr:twoCellAnchor>
-  <xdr:twoCellAnchor editAs="oneCell">
-    <xdr:from>
-      <xdr:col>5</xdr:col>
-      <xdr:colOff>111125</xdr:colOff>
-      <xdr:row>39</xdr:row>
-      <xdr:rowOff>79375</xdr:rowOff>
-    </xdr:from>
-    <xdr:to>
-      <xdr:col>17</xdr:col>
-      <xdr:colOff>644525</xdr:colOff>
-      <xdr:row>66</xdr:row>
-      <xdr:rowOff>147637</xdr:rowOff>
-    </xdr:to>
-    <xdr:pic>
-      <xdr:nvPicPr>
-        <xdr:cNvPr id="17" name="Image 16"/>
-        <xdr:cNvPicPr>
-          <a:picLocks noChangeAspect="1"/>
-        </xdr:cNvPicPr>
-      </xdr:nvPicPr>
-      <xdr:blipFill>
-        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId11">
-          <a:extLst>
-            <a:ext uri="{28A0092B-C50C-407E-A947-70E740481C1C}">
-              <a14:useLocalDpi xmlns:a14="http://schemas.microsoft.com/office/drawing/2010/main" val="0"/>
-            </a:ext>
-          </a:extLst>
-        </a:blip>
-        <a:stretch>
-          <a:fillRect/>
-        </a:stretch>
-      </xdr:blipFill>
-      <xdr:spPr>
-        <a:xfrm>
-          <a:off x="6477000" y="7239000"/>
-          <a:ext cx="10058400" cy="5029200"/>
-        </a:xfrm>
-        <a:prstGeom prst="rect">
-          <a:avLst/>
-        </a:prstGeom>
-      </xdr:spPr>
-    </xdr:pic>
-    <xdr:clientData/>
-  </xdr:twoCellAnchor>
-  <xdr:twoCellAnchor editAs="oneCell">
-    <xdr:from>
-      <xdr:col>11</xdr:col>
-      <xdr:colOff>7937</xdr:colOff>
-      <xdr:row>70</xdr:row>
-      <xdr:rowOff>15875</xdr:rowOff>
-    </xdr:from>
-    <xdr:to>
-      <xdr:col>16</xdr:col>
-      <xdr:colOff>626825</xdr:colOff>
-      <xdr:row>85</xdr:row>
-      <xdr:rowOff>164717</xdr:rowOff>
-    </xdr:to>
-    <xdr:pic>
-      <xdr:nvPicPr>
-        <xdr:cNvPr id="18" name="Image 17"/>
-        <xdr:cNvPicPr>
-          <a:picLocks noChangeAspect="1"/>
-        </xdr:cNvPicPr>
-      </xdr:nvPicPr>
-      <xdr:blipFill>
-        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId12">
-          <a:extLst>
-            <a:ext uri="{28A0092B-C50C-407E-A947-70E740481C1C}">
-              <a14:useLocalDpi xmlns:a14="http://schemas.microsoft.com/office/drawing/2010/main" val="0"/>
-            </a:ext>
-          </a:extLst>
-        </a:blip>
-        <a:stretch>
-          <a:fillRect/>
-        </a:stretch>
-      </xdr:blipFill>
-      <xdr:spPr>
-        <a:xfrm>
-          <a:off x="11136312" y="12866688"/>
-          <a:ext cx="4587638" cy="2911092"/>
-        </a:xfrm>
-        <a:prstGeom prst="rect">
-          <a:avLst/>
-        </a:prstGeom>
-      </xdr:spPr>
-    </xdr:pic>
-    <xdr:clientData/>
-  </xdr:twoCellAnchor>
-  <xdr:twoCellAnchor editAs="oneCell">
-    <xdr:from>
-      <xdr:col>5</xdr:col>
-      <xdr:colOff>0</xdr:colOff>
-      <xdr:row>87</xdr:row>
-      <xdr:rowOff>0</xdr:rowOff>
-    </xdr:from>
-    <xdr:to>
-      <xdr:col>15</xdr:col>
-      <xdr:colOff>308055</xdr:colOff>
-      <xdr:row>107</xdr:row>
-      <xdr:rowOff>74619</xdr:rowOff>
-    </xdr:to>
-    <xdr:pic>
-      <xdr:nvPicPr>
-        <xdr:cNvPr id="19" name="Image 18"/>
-        <xdr:cNvPicPr>
-          <a:picLocks noChangeAspect="1"/>
-        </xdr:cNvPicPr>
-      </xdr:nvPicPr>
-      <xdr:blipFill>
-        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId13">
-          <a:extLst>
-            <a:ext uri="{28A0092B-C50C-407E-A947-70E740481C1C}">
-              <a14:useLocalDpi xmlns:a14="http://schemas.microsoft.com/office/drawing/2010/main" val="0"/>
-            </a:ext>
-          </a:extLst>
-        </a:blip>
-        <a:stretch>
-          <a:fillRect/>
-        </a:stretch>
-      </xdr:blipFill>
-      <xdr:spPr>
-        <a:xfrm>
-          <a:off x="6596063" y="15986125"/>
-          <a:ext cx="8245555" cy="3741744"/>
-        </a:xfrm>
-        <a:prstGeom prst="rect">
-          <a:avLst/>
-        </a:prstGeom>
-      </xdr:spPr>
-    </xdr:pic>
-    <xdr:clientData/>
-  </xdr:twoCellAnchor>
-  <xdr:twoCellAnchor editAs="oneCell">
-    <xdr:from>
-      <xdr:col>10</xdr:col>
-      <xdr:colOff>762000</xdr:colOff>
-      <xdr:row>108</xdr:row>
-      <xdr:rowOff>47626</xdr:rowOff>
-    </xdr:from>
-    <xdr:to>
-      <xdr:col>18</xdr:col>
-      <xdr:colOff>214507</xdr:colOff>
-      <xdr:row>125</xdr:row>
-      <xdr:rowOff>6618</xdr:rowOff>
-    </xdr:to>
-    <xdr:pic>
-      <xdr:nvPicPr>
-        <xdr:cNvPr id="20" name="Image 19"/>
-        <xdr:cNvPicPr>
-          <a:picLocks noChangeAspect="1"/>
-        </xdr:cNvPicPr>
-      </xdr:nvPicPr>
-      <xdr:blipFill>
-        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId14">
-          <a:extLst>
-            <a:ext uri="{28A0092B-C50C-407E-A947-70E740481C1C}">
-              <a14:useLocalDpi xmlns:a14="http://schemas.microsoft.com/office/drawing/2010/main" val="0"/>
-            </a:ext>
-          </a:extLst>
-        </a:blip>
-        <a:stretch>
-          <a:fillRect/>
-        </a:stretch>
-      </xdr:blipFill>
-      <xdr:spPr>
-        <a:xfrm>
-          <a:off x="11326813" y="19883439"/>
-          <a:ext cx="5913632" cy="3086367"/>
-        </a:xfrm>
-        <a:prstGeom prst="rect">
-          <a:avLst/>
-        </a:prstGeom>
-      </xdr:spPr>
-    </xdr:pic>
-    <xdr:clientData/>
-  </xdr:twoCellAnchor>
-  <xdr:twoCellAnchor editAs="oneCell">
-    <xdr:from>
-      <xdr:col>5</xdr:col>
-      <xdr:colOff>182563</xdr:colOff>
-      <xdr:row>126</xdr:row>
-      <xdr:rowOff>23812</xdr:rowOff>
-    </xdr:from>
-    <xdr:to>
-      <xdr:col>13</xdr:col>
-      <xdr:colOff>211056</xdr:colOff>
-      <xdr:row>143</xdr:row>
-      <xdr:rowOff>66949</xdr:rowOff>
-    </xdr:to>
-    <xdr:pic>
-      <xdr:nvPicPr>
-        <xdr:cNvPr id="4" name="Image 3"/>
-        <xdr:cNvPicPr>
-          <a:picLocks noChangeAspect="1"/>
-        </xdr:cNvPicPr>
-      </xdr:nvPicPr>
-      <xdr:blipFill>
-        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId15">
-          <a:extLst>
-            <a:ext uri="{28A0092B-C50C-407E-A947-70E740481C1C}">
-              <a14:useLocalDpi xmlns:a14="http://schemas.microsoft.com/office/drawing/2010/main" val="0"/>
-            </a:ext>
-          </a:extLst>
-        </a:blip>
-        <a:stretch>
-          <a:fillRect/>
-        </a:stretch>
-      </xdr:blipFill>
-      <xdr:spPr>
-        <a:xfrm>
-          <a:off x="6778626" y="23177500"/>
-          <a:ext cx="6378493" cy="3162574"/>
         </a:xfrm>
         <a:prstGeom prst="rect">
           <a:avLst/>
@@ -2750,7 +2511,7 @@
         </xdr:cNvPicPr>
       </xdr:nvPicPr>
       <xdr:blipFill>
-        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId16">
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId9">
           <a:extLst>
             <a:ext uri="{28A0092B-C50C-407E-A947-70E740481C1C}">
               <a14:useLocalDpi xmlns:a14="http://schemas.microsoft.com/office/drawing/2010/main" val="0"/>
@@ -2794,7 +2555,7 @@
         </xdr:cNvPicPr>
       </xdr:nvPicPr>
       <xdr:blipFill>
-        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId17">
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId10">
           <a:extLst>
             <a:ext uri="{28A0092B-C50C-407E-A947-70E740481C1C}">
               <a14:useLocalDpi xmlns:a14="http://schemas.microsoft.com/office/drawing/2010/main" val="0"/>
@@ -2838,7 +2599,7 @@
         </xdr:cNvPicPr>
       </xdr:nvPicPr>
       <xdr:blipFill>
-        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId18">
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId11">
           <a:extLst>
             <a:ext uri="{28A0092B-C50C-407E-A947-70E740481C1C}">
               <a14:useLocalDpi xmlns:a14="http://schemas.microsoft.com/office/drawing/2010/main" val="0"/>
@@ -2882,7 +2643,7 @@
         </xdr:cNvPicPr>
       </xdr:nvPicPr>
       <xdr:blipFill>
-        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId19">
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId12">
           <a:extLst>
             <a:ext uri="{28A0092B-C50C-407E-A947-70E740481C1C}">
               <a14:useLocalDpi xmlns:a14="http://schemas.microsoft.com/office/drawing/2010/main" val="0"/>
@@ -3360,13 +3121,13 @@
         <v>13</v>
       </c>
       <c r="B42" s="5" t="s">
-        <v>122</v>
+        <v>124</v>
       </c>
       <c r="C42" s="2" t="s">
-        <v>49</v>
+        <v>125</v>
       </c>
       <c r="D42" s="2" t="s">
-        <v>48</v>
+        <v>126</v>
       </c>
       <c r="E42" s="2" t="s">
         <v>127</v>
@@ -3377,16 +3138,16 @@
         <v>14</v>
       </c>
       <c r="B43" s="5" t="s">
-        <v>123</v>
+        <v>128</v>
       </c>
       <c r="C43" s="3" t="s">
-        <v>124</v>
+        <v>129</v>
       </c>
       <c r="D43" s="3" t="s">
-        <v>125</v>
+        <v>130</v>
       </c>
       <c r="E43" s="3" t="s">
-        <v>126</v>
+        <v>131</v>
       </c>
     </row>
     <row r="71" spans="1:5" ht="15" thickBot="1" x14ac:dyDescent="0.35"/>
@@ -3412,7 +3173,7 @@
         <v>16</v>
       </c>
       <c r="B73" s="5" t="s">
-        <v>15</v>
+        <v>123</v>
       </c>
       <c r="C73" s="3" t="s">
         <v>54</v>
@@ -3421,7 +3182,7 @@
         <v>53</v>
       </c>
       <c r="E73" s="3" t="s">
-        <v>52</v>
+        <v>122</v>
       </c>
     </row>
     <row r="74" spans="1:5" x14ac:dyDescent="0.3">
@@ -3451,16 +3212,16 @@
         <v>20</v>
       </c>
       <c r="B89" s="11" t="s">
-        <v>17</v>
+        <v>132</v>
       </c>
       <c r="C89" s="7">
         <v>0</v>
       </c>
       <c r="D89" s="7" t="s">
-        <v>55</v>
+        <v>133</v>
       </c>
       <c r="E89" s="16" t="s">
-        <v>56</v>
+        <v>134</v>
       </c>
     </row>
     <row r="90" spans="1:5" x14ac:dyDescent="0.3">
@@ -3468,16 +3229,16 @@
         <v>21</v>
       </c>
       <c r="B90" s="12" t="s">
-        <v>18</v>
+        <v>135</v>
       </c>
       <c r="C90" s="2" t="s">
-        <v>57</v>
+        <v>136</v>
       </c>
       <c r="D90" s="2" t="s">
-        <v>58</v>
+        <v>137</v>
       </c>
       <c r="E90" s="17" t="s">
-        <v>59</v>
+        <v>138</v>
       </c>
     </row>
     <row r="91" spans="1:5" ht="15" thickBot="1" x14ac:dyDescent="0.35">
@@ -3485,16 +3246,16 @@
         <v>22</v>
       </c>
       <c r="B91" s="13" t="s">
-        <v>19</v>
+        <v>139</v>
       </c>
       <c r="C91" s="3" t="s">
-        <v>60</v>
+        <v>140</v>
       </c>
       <c r="D91" s="3" t="s">
-        <v>61</v>
+        <v>141</v>
       </c>
       <c r="E91" s="18" t="s">
-        <v>62</v>
+        <v>142</v>
       </c>
     </row>
     <row r="110" spans="1:5" ht="15" thickBot="1" x14ac:dyDescent="0.35"/>
@@ -3520,16 +3281,16 @@
         <v>63</v>
       </c>
       <c r="B112" s="5" t="s">
-        <v>23</v>
+        <v>143</v>
       </c>
       <c r="C112" s="19" t="s">
-        <v>64</v>
+        <v>144</v>
       </c>
       <c r="D112" s="19" t="s">
-        <v>65</v>
+        <v>145</v>
       </c>
       <c r="E112" s="20" t="s">
-        <v>66</v>
+        <v>146</v>
       </c>
     </row>
     <row r="126" spans="1:18" ht="15" thickBot="1" x14ac:dyDescent="0.35"/>
@@ -3555,16 +3316,16 @@
         <v>71</v>
       </c>
       <c r="B128" s="5" t="s">
-        <v>67</v>
+        <v>147</v>
       </c>
       <c r="C128" s="19" t="s">
-        <v>68</v>
+        <v>148</v>
       </c>
       <c r="D128" s="19" t="s">
-        <v>69</v>
+        <v>149</v>
       </c>
       <c r="E128" s="20" t="s">
-        <v>70</v>
+        <v>150</v>
       </c>
       <c r="R128" t="s">
         <v>72</v>

</xml_diff>